<commit_message>
tmp: Refine PEB test UI, scenario sources and persistent reports
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
+++ b/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\tests\PersonalEventBuilder\Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65DAFC7D-FA89-4600-9C0F-436C9C229FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{570194B4-5804-4A7E-A871-96F650668B92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
     <definedName name="_Hlk209437159" localSheetId="0">'5. Тимчасово відсутні'!#REF!</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Т (Х)'!$A$1:$BQ$30</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="manual"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="171">
   <si>
     <t>Індекс посади</t>
   </si>
@@ -134,9 +134,6 @@
     <t>Відпустка</t>
   </si>
   <si>
-    <t>солдат</t>
-  </si>
-  <si>
     <t>Підрозділи</t>
   </si>
   <si>
@@ -413,12 +410,6 @@
     <t>ПРИКОМАНДИРОВАНІ</t>
   </si>
   <si>
-    <t>№296</t>
-  </si>
-  <si>
-    <t>№120</t>
-  </si>
-  <si>
     <t>311 ЗАПАСНА РОТА</t>
   </si>
   <si>
@@ -518,18 +509,6 @@
     <t>76</t>
   </si>
   <si>
-    <t>лейтенант</t>
-  </si>
-  <si>
-    <t>?</t>
-  </si>
-  <si>
-    <t>Самовільне залишення частини</t>
-  </si>
-  <si>
-    <t>Відпустка для лікування</t>
-  </si>
-  <si>
     <t>71 (А)</t>
   </si>
   <si>
@@ -587,22 +566,7 @@
     <t>Стовпець2</t>
   </si>
   <si>
-    <t>А4862</t>
-  </si>
-  <si>
     <t>Стовпець3</t>
-  </si>
-  <si>
-    <t>ВАСИЛЕНКО Ростислав Євгенійович</t>
-  </si>
-  <si>
-    <t>A1A0098</t>
-  </si>
-  <si>
-    <t>повідомлення командира військової частини А4862 № 2456/36526 від 21.04.2026 (вх. № 5806 від 22.04.2026), посвідчення про відрядження № 3/71/2659 від 24.04.2026;</t>
-  </si>
-  <si>
-    <t>СЗЧ, ПРИБУВ, (7401)</t>
   </si>
   <si>
     <r>
@@ -666,16 +630,13 @@
     </r>
   </si>
   <si>
-    <t>м. Харків, Харківська обл.</t>
-  </si>
-  <si>
-    <t>ПЕРЕБУВАВ на лікуванні, відпускний квиток № 2026/296/7 від 13.10.2026</t>
-  </si>
-  <si>
     <t>БОНДАРЕНКО Олександр Юрійович</t>
   </si>
   <si>
-    <t>В00К3252</t>
+    <t>Щорічна відпустка</t>
+  </si>
+  <si>
+    <t>м. Тестоград</t>
   </si>
 </sst>
 </file>
@@ -683,10 +644,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="000000"/>
-    <numFmt numFmtId="165" formatCode="mmmm\ yyyy"/>
+    <numFmt numFmtId="164" formatCode="mmmm\ yyyy"/>
+    <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="44" x14ac:knownFonts="1">
+  <fonts count="47" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -953,12 +914,6 @@
     </font>
     <font>
       <sz val="14"/>
-      <color theme="0"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="14"/>
       <color theme="5" tint="0.39997558519241921"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -999,8 +954,28 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="5" tint="0.39997558519241921"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFADADAD"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF00B050"/>
+      <name val="Times New Roman"/>
+    </font>
   </fonts>
-  <fills count="22">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1016,12 +991,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1092,12 +1061,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF404040"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1115,7 +1078,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="63">
+  <borders count="62">
     <border>
       <left/>
       <right/>
@@ -1773,17 +1736,6 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1898,111 +1850,111 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="55" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="57" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="55" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="57" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="59" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="60" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="59" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="17" borderId="61" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="62" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="60" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="61" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="55" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="57" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="55" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="57" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="59" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="60" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="59" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="17" borderId="61" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="62" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="60" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="61" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="55" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="57" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="55" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="57" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="59" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="60" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="59" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="17" borderId="61" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="62" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="60" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="61" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="55" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="57" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="55" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="57" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="59" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="60" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="59" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="17" borderId="61" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="62" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="60" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="61" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
@@ -2035,31 +1987,31 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="55" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="59" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="60" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="54" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="58" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="59" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="17" borderId="61" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="62" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="60" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="61" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="1">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="154">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
@@ -2198,25 +2150,16 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="39" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="38" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2225,167 +2168,104 @@
     <xf numFmtId="14" fontId="36" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="36" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="36" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="36" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="50" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="36" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="36" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="36" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="36" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="39" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="35" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="40" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="38" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="18" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="40" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="40" fillId="18" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="38" fillId="18" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="36" fillId="19" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="43" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="35" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="41" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="43" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="39" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="40" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="40" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="43" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="44" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="43" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="43" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="43" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="45" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="46" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="36" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="43" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="36" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="36" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="20" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="41" fillId="20" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="39" fillId="20" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="36" fillId="21" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="39" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="38" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2672,7 +2552,7 @@
     <cellStyle name="Хороший 4" xfId="107" xr:uid="{00000000-0005-0000-0000-00009F000000}"/>
     <cellStyle name="Хороший 5" xfId="25" xr:uid="{00000000-0005-0000-0000-0000A0000000}"/>
   </cellStyles>
-  <dxfs count="41">
+  <dxfs count="34">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2680,76 +2560,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2799,7 +2609,7 @@
         <name val="Times New Roman"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -2836,7 +2646,7 @@
         <name val="Times New Roman"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -2952,7 +2762,7 @@
         <name val="Times New Roman"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -2991,7 +2801,7 @@
         <name val="Times New Roman"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -3030,7 +2840,7 @@
         <name val="Times New Roman"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -3069,7 +2879,7 @@
         <name val="Times New Roman"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -3147,7 +2957,7 @@
         <name val="Times New Roman"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -3186,7 +2996,7 @@
         <name val="Times New Roman"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -3225,7 +3035,7 @@
         <name val="Times New Roman"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -3620,14 +3430,14 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="TableStyleDark_my" pivot="0" count="8" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="40"/>
-      <tableStyleElement type="headerRow" dxfId="39"/>
-      <tableStyleElement type="totalRow" dxfId="38"/>
-      <tableStyleElement type="firstColumn" dxfId="37"/>
-      <tableStyleElement type="lastColumn" dxfId="36"/>
-      <tableStyleElement type="firstRowStripe" dxfId="35"/>
-      <tableStyleElement type="secondRowStripe" dxfId="34"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="33"/>
+      <tableStyleElement type="wholeTable" dxfId="33"/>
+      <tableStyleElement type="headerRow" dxfId="32"/>
+      <tableStyleElement type="totalRow" dxfId="31"/>
+      <tableStyleElement type="firstColumn" dxfId="30"/>
+      <tableStyleElement type="lastColumn" dxfId="29"/>
+      <tableStyleElement type="firstRowStripe" dxfId="28"/>
+      <tableStyleElement type="secondRowStripe" dxfId="27"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="26"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -3648,28 +3458,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="ВІДСУТНІ" displayName="ВІДСУТНІ" ref="A5:Q29" totalsRowShown="0" headerRowDxfId="32" dataDxfId="30" headerRowBorderDxfId="31" tableBorderDxfId="29" totalsRowBorderDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="ВІДСУТНІ" displayName="ВІДСУТНІ" ref="A5:Q9" totalsRowShown="0" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24" tableBorderDxfId="22" totalsRowBorderDxfId="21">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:P5">
     <sortCondition ref="G5"/>
   </sortState>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="65" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="66" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="67" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="68" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="69" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="70" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="71 (А)" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="71 (Б)" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="72" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="73" dataDxfId="18"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="74" dataDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="75 (А)" dataDxfId="16"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0300-00000D000000}" name="75 (Б)" dataDxfId="15"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0300-00000E000000}" name="76" dataDxfId="14"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0300-00000F000000}" name="Стовпець1" dataDxfId="13"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0300-000010000000}" name="Стовпець2" dataDxfId="12"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0300-000011000000}" name="Стовпець3" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="65" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="66" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="67" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="68" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="69" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="70" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="71 (А)" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="71 (Б)" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="72" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="73" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="74" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="75 (А)" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0300-00000D000000}" name="75 (Б)" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0300-00000E000000}" name="76" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0300-00000F000000}" name="Стовпець1" dataDxfId="6"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0300-000010000000}" name="Стовпець2" dataDxfId="5"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0300-000011000000}" name="Стовпець3" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark_my" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3996,718 +3806,262 @@
     <tabColor rgb="FFFF0000"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" style="84" customWidth="1"/>
-    <col min="2" max="2" width="37.28515625" style="84" customWidth="1"/>
-    <col min="3" max="3" width="16.85546875" style="84" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" style="84" customWidth="1"/>
-    <col min="5" max="5" width="41.85546875" style="84" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" style="84" customWidth="1"/>
-    <col min="7" max="7" width="16" style="84" customWidth="1"/>
-    <col min="8" max="8" width="9.85546875" style="84" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" style="84" customWidth="1"/>
-    <col min="10" max="10" width="15.7109375" style="84" customWidth="1"/>
-    <col min="11" max="11" width="16.28515625" style="84" customWidth="1"/>
-    <col min="12" max="12" width="14.42578125" style="84" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="84" customWidth="1"/>
-    <col min="14" max="14" width="47.85546875" style="84" customWidth="1"/>
-    <col min="15" max="15" width="15.85546875" style="84" customWidth="1"/>
-    <col min="16" max="16" width="14.85546875" style="84" customWidth="1"/>
-    <col min="17" max="17" width="24.5703125" style="84" customWidth="1"/>
-    <col min="18" max="16384" width="8.85546875" style="84"/>
+    <col min="1" max="1" width="20.85546875" style="60" customWidth="1"/>
+    <col min="2" max="2" width="37.28515625" style="60" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" style="60" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" style="60" customWidth="1"/>
+    <col min="5" max="5" width="41.85546875" style="60" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" style="60" customWidth="1"/>
+    <col min="7" max="7" width="16" style="60" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" style="60" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" style="60" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" style="60" customWidth="1"/>
+    <col min="11" max="11" width="16.28515625" style="60" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" style="60" customWidth="1"/>
+    <col min="13" max="13" width="14.28515625" style="60" customWidth="1"/>
+    <col min="14" max="14" width="47.85546875" style="60" customWidth="1"/>
+    <col min="15" max="15" width="15.85546875" style="60" customWidth="1"/>
+    <col min="16" max="16" width="14.85546875" style="60" customWidth="1"/>
+    <col min="17" max="17" width="24.5703125" style="60" customWidth="1"/>
+    <col min="18" max="16384" width="8.85546875" style="60"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="52" customFormat="1" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="111"/>
-      <c r="B1" s="111"/>
-      <c r="C1" s="111"/>
-      <c r="D1" s="111"/>
-      <c r="E1" s="111"/>
-      <c r="F1" s="111"/>
-      <c r="G1" s="111"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="111"/>
-      <c r="J1" s="111"/>
-      <c r="K1" s="111"/>
-      <c r="L1" s="111"/>
-      <c r="M1" s="111"/>
-      <c r="N1" s="111"/>
+    <row r="1" spans="1:17" s="49" customFormat="1" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="87"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
+      <c r="I1" s="87"/>
+      <c r="J1" s="87"/>
+      <c r="K1" s="87"/>
+      <c r="L1" s="87"/>
+      <c r="M1" s="87"/>
+      <c r="N1" s="87"/>
     </row>
-    <row r="2" spans="1:17" s="86" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="53">
+    <row r="2" spans="1:17" s="62" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="50">
         <v>45772</v>
       </c>
-      <c r="B2" s="112" t="s">
+      <c r="B2" s="88" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="112"/>
-      <c r="D2" s="112"/>
-      <c r="E2" s="112"/>
-      <c r="F2" s="112"/>
-      <c r="G2" s="112"/>
-      <c r="H2" s="112"/>
-      <c r="I2" s="112"/>
-      <c r="J2" s="112"/>
-      <c r="K2" s="112"/>
-      <c r="L2" s="112"/>
-      <c r="M2" s="112"/>
-      <c r="N2" s="112"/>
-      <c r="O2" s="85"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="88"/>
+      <c r="E2" s="88"/>
+      <c r="F2" s="88"/>
+      <c r="G2" s="88"/>
+      <c r="H2" s="88"/>
+      <c r="I2" s="88"/>
+      <c r="J2" s="88"/>
+      <c r="K2" s="88"/>
+      <c r="L2" s="88"/>
+      <c r="M2" s="88"/>
+      <c r="N2" s="88"/>
+      <c r="O2" s="61"/>
     </row>
-    <row r="3" spans="1:17" s="86" customFormat="1" ht="117.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="54" t="s">
+    <row r="3" spans="1:17" s="62" customFormat="1" ht="117.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="54" t="s">
+      <c r="C3" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="87" t="s">
-        <v>177</v>
-      </c>
-      <c r="E3" s="88" t="s">
+      <c r="D3" s="63" t="s">
+        <v>165</v>
+      </c>
+      <c r="E3" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="88" t="s">
+      <c r="F3" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="113" t="s">
+      <c r="G3" s="89" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="113"/>
-      <c r="I3" s="87" t="s">
-        <v>178</v>
-      </c>
-      <c r="J3" s="88" t="s">
-        <v>179</v>
-      </c>
-      <c r="K3" s="88" t="s">
+      <c r="H3" s="89"/>
+      <c r="I3" s="63" t="s">
+        <v>166</v>
+      </c>
+      <c r="J3" s="64" t="s">
+        <v>167</v>
+      </c>
+      <c r="K3" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="113" t="s">
+      <c r="L3" s="89" t="s">
         <v>12</v>
       </c>
-      <c r="M3" s="113"/>
-      <c r="N3" s="88" t="s">
+      <c r="M3" s="89"/>
+      <c r="N3" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="O3" s="85"/>
+      <c r="O3" s="61"/>
     </row>
-    <row r="4" spans="1:17" s="86" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="105"/>
-      <c r="B4" s="110"/>
-      <c r="C4" s="106"/>
-      <c r="D4" s="107"/>
-      <c r="E4" s="108"/>
-      <c r="F4" s="108"/>
-      <c r="G4" s="108"/>
-      <c r="H4" s="108"/>
-      <c r="I4" s="107"/>
-      <c r="J4" s="108"/>
-      <c r="K4" s="108"/>
-      <c r="L4" s="108"/>
-      <c r="M4" s="108"/>
-      <c r="N4" s="108"/>
-      <c r="O4" s="109"/>
+    <row r="4" spans="1:17" s="62" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="70"/>
+      <c r="B4" s="75"/>
+      <c r="C4" s="71"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="72"/>
+      <c r="J4" s="73"/>
+      <c r="K4" s="73"/>
+      <c r="L4" s="73"/>
+      <c r="M4" s="73"/>
+      <c r="N4" s="73"/>
+      <c r="O4" s="74"/>
     </row>
     <row r="5" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="101" t="s">
+      <c r="A5" s="66" t="s">
+        <v>135</v>
+      </c>
+      <c r="B5" s="67" t="s">
+        <v>136</v>
+      </c>
+      <c r="C5" s="67" t="s">
+        <v>137</v>
+      </c>
+      <c r="D5" s="67" t="s">
         <v>138</v>
       </c>
-      <c r="B5" s="102" t="s">
+      <c r="E5" s="67" t="s">
         <v>139</v>
       </c>
-      <c r="C5" s="102" t="s">
+      <c r="F5" s="67" t="s">
         <v>140</v>
       </c>
-      <c r="D5" s="102" t="s">
+      <c r="G5" s="67" t="s">
+        <v>145</v>
+      </c>
+      <c r="H5" s="67" t="s">
+        <v>146</v>
+      </c>
+      <c r="I5" s="67" t="s">
         <v>141</v>
       </c>
-      <c r="E5" s="102" t="s">
+      <c r="J5" s="67" t="s">
         <v>142</v>
       </c>
-      <c r="F5" s="102" t="s">
+      <c r="K5" s="67" t="s">
         <v>143</v>
       </c>
-      <c r="G5" s="102" t="s">
-        <v>152</v>
-      </c>
-      <c r="H5" s="102" t="s">
-        <v>153</v>
-      </c>
-      <c r="I5" s="102" t="s">
+      <c r="L5" s="67" t="s">
+        <v>147</v>
+      </c>
+      <c r="M5" s="67" t="s">
+        <v>148</v>
+      </c>
+      <c r="N5" s="67" t="s">
         <v>144</v>
       </c>
-      <c r="J5" s="102" t="s">
-        <v>145</v>
-      </c>
-      <c r="K5" s="102" t="s">
-        <v>146</v>
-      </c>
-      <c r="L5" s="102" t="s">
-        <v>154</v>
-      </c>
-      <c r="M5" s="102" t="s">
-        <v>155</v>
-      </c>
-      <c r="N5" s="102" t="s">
-        <v>147</v>
-      </c>
-      <c r="O5" s="103" t="s">
-        <v>169</v>
-      </c>
-      <c r="P5" s="102" t="s">
-        <v>170</v>
-      </c>
-      <c r="Q5" s="104" t="s">
-        <v>172</v>
+      <c r="O5" s="68" t="s">
+        <v>162</v>
+      </c>
+      <c r="P5" s="67" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q5" s="69" t="s">
+        <v>164</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="72" t="s">
-        <v>148</v>
-      </c>
-      <c r="B6" s="60" t="s">
-        <v>182</v>
-      </c>
-      <c r="C6" s="58" t="s">
-        <v>183</v>
-      </c>
-      <c r="D6" s="51" t="s">
-        <v>151</v>
-      </c>
-      <c r="E6" s="51" t="s">
-        <v>180</v>
-      </c>
-      <c r="F6" s="56">
-        <v>46309</v>
-      </c>
-      <c r="G6" s="56">
-        <v>46308</v>
-      </c>
-      <c r="H6" s="56" t="s">
-        <v>113</v>
-      </c>
-      <c r="I6" s="78">
-        <v>30</v>
-      </c>
-      <c r="J6" s="80">
-        <v>46339</v>
-      </c>
-      <c r="K6" s="56"/>
-      <c r="L6" s="56"/>
-      <c r="M6" s="56"/>
-      <c r="N6" s="78" t="s">
-        <v>181</v>
-      </c>
-      <c r="O6" s="55">
-        <v>7</v>
-      </c>
-      <c r="P6" s="91"/>
-      <c r="Q6" s="61"/>
+    <row r="6" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="57"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="53"/>
+      <c r="I6" s="58"/>
+      <c r="J6" s="59"/>
+      <c r="K6" s="53"/>
+      <c r="L6" s="53"/>
+      <c r="M6" s="53"/>
+      <c r="N6" s="58"/>
+      <c r="O6" s="52"/>
+      <c r="P6" s="65"/>
+      <c r="Q6" s="56"/>
     </row>
     <row r="7" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="72"/>
-      <c r="B7" s="60"/>
-      <c r="C7" s="58"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="56"/>
-      <c r="G7" s="56"/>
-      <c r="H7" s="56"/>
-      <c r="I7" s="78"/>
-      <c r="J7" s="80"/>
-      <c r="K7" s="56"/>
-      <c r="L7" s="56"/>
-      <c r="M7" s="56"/>
-      <c r="N7" s="78"/>
-      <c r="O7" s="55"/>
-      <c r="P7" s="91"/>
-      <c r="Q7" s="61"/>
+      <c r="A7" s="57"/>
+      <c r="B7" s="55"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="53"/>
+      <c r="G7" s="53"/>
+      <c r="H7" s="53"/>
+      <c r="I7" s="58"/>
+      <c r="J7" s="59"/>
+      <c r="K7" s="53"/>
+      <c r="L7" s="53"/>
+      <c r="M7" s="53"/>
+      <c r="N7" s="58"/>
+      <c r="O7" s="52"/>
+      <c r="P7" s="65"/>
+      <c r="Q7" s="56"/>
     </row>
     <row r="8" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="72"/>
-      <c r="B8" s="60"/>
-      <c r="C8" s="58"/>
-      <c r="D8" s="51"/>
-      <c r="E8" s="51"/>
-      <c r="F8" s="56"/>
-      <c r="G8" s="56"/>
-      <c r="H8" s="56"/>
-      <c r="I8" s="78"/>
-      <c r="J8" s="80"/>
-      <c r="K8" s="56"/>
-      <c r="L8" s="56"/>
-      <c r="M8" s="56"/>
-      <c r="N8" s="78"/>
-      <c r="O8" s="55"/>
-      <c r="P8" s="91"/>
-      <c r="Q8" s="61"/>
+      <c r="A8" s="57"/>
+      <c r="B8" s="55"/>
+      <c r="C8" s="54"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="53"/>
+      <c r="G8" s="53"/>
+      <c r="H8" s="53"/>
+      <c r="I8" s="58"/>
+      <c r="J8" s="59"/>
+      <c r="K8" s="53"/>
+      <c r="L8" s="53"/>
+      <c r="M8" s="53"/>
+      <c r="N8" s="58"/>
+      <c r="O8" s="52"/>
+      <c r="P8" s="65"/>
+      <c r="Q8" s="56"/>
     </row>
-    <row r="9" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="72"/>
-      <c r="B9" s="60"/>
-      <c r="C9" s="58"/>
-      <c r="D9" s="51"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="56"/>
-      <c r="G9" s="56"/>
-      <c r="H9" s="56"/>
-      <c r="I9" s="78"/>
-      <c r="J9" s="80"/>
-      <c r="K9" s="56"/>
-      <c r="L9" s="56"/>
-      <c r="M9" s="56"/>
-      <c r="N9" s="78"/>
-      <c r="O9" s="55"/>
-      <c r="P9" s="91"/>
-      <c r="Q9" s="61"/>
-    </row>
-    <row r="10" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="72"/>
-      <c r="B10" s="60"/>
-      <c r="C10" s="58"/>
-      <c r="D10" s="51"/>
-      <c r="E10" s="51"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
-      <c r="H10" s="56"/>
-      <c r="I10" s="78"/>
-      <c r="J10" s="80"/>
-      <c r="K10" s="56"/>
-      <c r="L10" s="56"/>
-      <c r="M10" s="56"/>
-      <c r="N10" s="78"/>
-      <c r="O10" s="55"/>
-      <c r="P10" s="91"/>
-      <c r="Q10" s="61"/>
-    </row>
-    <row r="11" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="72"/>
-      <c r="B11" s="60"/>
-      <c r="C11" s="58"/>
-      <c r="D11" s="51"/>
-      <c r="E11" s="51"/>
-      <c r="F11" s="56"/>
-      <c r="G11" s="56"/>
-      <c r="H11" s="56"/>
-      <c r="I11" s="78"/>
-      <c r="J11" s="80"/>
-      <c r="K11" s="56"/>
-      <c r="L11" s="56"/>
-      <c r="M11" s="56"/>
-      <c r="N11" s="78"/>
-      <c r="O11" s="55"/>
-      <c r="P11" s="91"/>
-      <c r="Q11" s="61"/>
-    </row>
-    <row r="12" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="72"/>
-      <c r="B12" s="60"/>
-      <c r="C12" s="58"/>
-      <c r="D12" s="51"/>
-      <c r="E12" s="51"/>
-      <c r="F12" s="56"/>
-      <c r="G12" s="56"/>
-      <c r="H12" s="56"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="80"/>
-      <c r="K12" s="56"/>
-      <c r="L12" s="56"/>
-      <c r="M12" s="56"/>
-      <c r="N12" s="78"/>
-      <c r="O12" s="55"/>
-      <c r="P12" s="91"/>
-      <c r="Q12" s="61"/>
-    </row>
-    <row r="13" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="72"/>
-      <c r="B13" s="60"/>
-      <c r="C13" s="58"/>
-      <c r="D13" s="51"/>
-      <c r="E13" s="51"/>
-      <c r="F13" s="56"/>
-      <c r="G13" s="56"/>
-      <c r="H13" s="56"/>
-      <c r="I13" s="78"/>
-      <c r="J13" s="80"/>
-      <c r="K13" s="56"/>
-      <c r="L13" s="56"/>
-      <c r="M13" s="56"/>
-      <c r="N13" s="78"/>
-      <c r="O13" s="55"/>
-      <c r="P13" s="91"/>
-      <c r="Q13" s="61"/>
-    </row>
-    <row r="14" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="72"/>
-      <c r="B14" s="60"/>
-      <c r="C14" s="58"/>
-      <c r="D14" s="51"/>
-      <c r="E14" s="51"/>
-      <c r="F14" s="56"/>
-      <c r="G14" s="56"/>
-      <c r="H14" s="56"/>
-      <c r="I14" s="78"/>
-      <c r="J14" s="80"/>
-      <c r="K14" s="56"/>
-      <c r="L14" s="56"/>
-      <c r="M14" s="56"/>
-      <c r="N14" s="78"/>
-      <c r="O14" s="55"/>
-      <c r="P14" s="91"/>
-      <c r="Q14" s="61"/>
-    </row>
-    <row r="15" spans="1:17" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A15" s="98" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="50" t="s">
-        <v>173</v>
-      </c>
-      <c r="C15" s="75" t="s">
-        <v>174</v>
-      </c>
-      <c r="D15" s="77" t="s">
-        <v>150</v>
-      </c>
-      <c r="E15" s="77" t="s">
-        <v>149</v>
-      </c>
-      <c r="F15" s="57">
-        <v>45393</v>
-      </c>
-      <c r="G15" s="69">
-        <v>46136</v>
-      </c>
-      <c r="H15" s="69" t="s">
-        <v>114</v>
-      </c>
-      <c r="I15" s="78" t="s">
-        <v>149</v>
-      </c>
-      <c r="J15" s="80" t="s">
-        <v>149</v>
-      </c>
-      <c r="K15" s="69">
-        <v>46129</v>
-      </c>
-      <c r="L15" s="69">
-        <v>46136</v>
-      </c>
-      <c r="M15" s="69" t="s">
-        <v>114</v>
-      </c>
-      <c r="N15" s="78" t="s">
-        <v>176</v>
-      </c>
-      <c r="O15" s="55"/>
-      <c r="P15" s="91"/>
-      <c r="Q15" s="96"/>
-    </row>
-    <row r="16" spans="1:17" ht="93.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="97" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="73" t="s">
-        <v>173</v>
-      </c>
-      <c r="C16" s="74" t="s">
-        <v>174</v>
-      </c>
-      <c r="D16" s="77" t="s">
-        <v>27</v>
-      </c>
-      <c r="E16" s="77" t="s">
-        <v>171</v>
-      </c>
-      <c r="F16" s="69">
-        <v>46136</v>
-      </c>
-      <c r="G16" s="69">
-        <v>46136</v>
-      </c>
-      <c r="H16" s="69" t="s">
-        <v>114</v>
-      </c>
-      <c r="I16" s="83" t="s">
-        <v>149</v>
-      </c>
-      <c r="J16" s="90" t="s">
-        <v>149</v>
-      </c>
-      <c r="K16" s="69"/>
-      <c r="L16" s="69"/>
-      <c r="M16" s="69"/>
-      <c r="N16" s="83" t="s">
-        <v>175</v>
-      </c>
-      <c r="O16" s="55"/>
-      <c r="P16" s="93" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q16" s="96"/>
-    </row>
-    <row r="17" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="95"/>
-      <c r="B17" s="48"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="51"/>
-      <c r="E17" s="51"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="56"/>
-      <c r="I17" s="78"/>
-      <c r="J17" s="80"/>
-      <c r="K17" s="56"/>
-      <c r="L17" s="56"/>
-      <c r="M17" s="56"/>
-      <c r="N17" s="78"/>
-      <c r="O17" s="55"/>
-      <c r="P17" s="92"/>
-      <c r="Q17" s="96"/>
-    </row>
-    <row r="18" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="72"/>
-      <c r="B18" s="60"/>
-      <c r="C18" s="58"/>
-      <c r="D18" s="51"/>
-      <c r="E18" s="51"/>
-      <c r="F18" s="56"/>
-      <c r="G18" s="56"/>
-      <c r="H18" s="56"/>
-      <c r="I18" s="78"/>
-      <c r="J18" s="80"/>
-      <c r="K18" s="56"/>
-      <c r="L18" s="56"/>
-      <c r="M18" s="56"/>
-      <c r="N18" s="78"/>
-      <c r="O18" s="55"/>
-      <c r="P18" s="92"/>
-      <c r="Q18" s="96"/>
-    </row>
-    <row r="19" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="72"/>
-      <c r="B19" s="60"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="51"/>
-      <c r="E19" s="51"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="56"/>
-      <c r="H19" s="56"/>
-      <c r="I19" s="78"/>
-      <c r="J19" s="80"/>
-      <c r="K19" s="56"/>
-      <c r="L19" s="56"/>
-      <c r="M19" s="56"/>
-      <c r="N19" s="78"/>
-      <c r="O19" s="55"/>
-      <c r="P19" s="92"/>
-      <c r="Q19" s="96"/>
-    </row>
-    <row r="20" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="95"/>
-      <c r="B20" s="65"/>
-      <c r="C20" s="49"/>
-      <c r="D20" s="51"/>
-      <c r="E20" s="51"/>
-      <c r="F20" s="56"/>
-      <c r="G20" s="56"/>
-      <c r="H20" s="56"/>
-      <c r="I20" s="78"/>
-      <c r="J20" s="80"/>
-      <c r="K20" s="56"/>
-      <c r="L20" s="56"/>
-      <c r="M20" s="56"/>
-      <c r="N20" s="78"/>
-      <c r="O20" s="55"/>
-      <c r="P20" s="92"/>
-      <c r="Q20" s="96"/>
-    </row>
-    <row r="21" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="72"/>
-      <c r="B21" s="60"/>
-      <c r="C21" s="58"/>
-      <c r="D21" s="51"/>
-      <c r="E21" s="51"/>
-      <c r="F21" s="56"/>
-      <c r="G21" s="56"/>
-      <c r="H21" s="56"/>
-      <c r="I21" s="78"/>
-      <c r="J21" s="80"/>
-      <c r="K21" s="56"/>
-      <c r="L21" s="56"/>
-      <c r="M21" s="56"/>
-      <c r="N21" s="78"/>
-      <c r="O21" s="55"/>
-      <c r="P21" s="92"/>
-      <c r="Q21" s="96"/>
-    </row>
-    <row r="22" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="72"/>
-      <c r="B22" s="60"/>
-      <c r="C22" s="58"/>
-      <c r="D22" s="51"/>
-      <c r="E22" s="51"/>
-      <c r="F22" s="56"/>
-      <c r="G22" s="56"/>
-      <c r="H22" s="56"/>
-      <c r="I22" s="78"/>
-      <c r="J22" s="80"/>
-      <c r="K22" s="56"/>
-      <c r="L22" s="56"/>
-      <c r="M22" s="71">
-        <v>2026</v>
-      </c>
-      <c r="N22" s="82">
-        <v>1042</v>
-      </c>
-      <c r="O22" s="55"/>
-      <c r="P22" s="92"/>
-      <c r="Q22" s="96"/>
-    </row>
-    <row r="23" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="95"/>
-      <c r="B23" s="48"/>
-      <c r="C23" s="67"/>
-      <c r="D23" s="51"/>
-      <c r="E23" s="51"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="78"/>
-      <c r="J23" s="80"/>
-      <c r="K23" s="56"/>
-      <c r="L23" s="56"/>
-      <c r="M23" s="70"/>
-      <c r="N23" s="82">
-        <v>2742</v>
-      </c>
-      <c r="O23" s="55"/>
-      <c r="P23" s="92"/>
-      <c r="Q23" s="96"/>
-    </row>
-    <row r="24" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="95"/>
-      <c r="B24" s="48"/>
-      <c r="C24" s="64"/>
-      <c r="D24" s="51"/>
-      <c r="E24" s="51"/>
-      <c r="F24" s="56"/>
-      <c r="G24" s="56"/>
-      <c r="H24" s="56"/>
-      <c r="I24" s="78"/>
-      <c r="J24" s="80"/>
-      <c r="K24" s="56"/>
-      <c r="L24" s="56"/>
-      <c r="M24" s="70"/>
-      <c r="N24" s="82">
-        <v>2659</v>
-      </c>
-      <c r="O24" s="55"/>
-      <c r="P24" s="92"/>
-      <c r="Q24" s="96"/>
-    </row>
-    <row r="25" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="72"/>
-      <c r="B25" s="60"/>
-      <c r="C25" s="58"/>
-      <c r="D25" s="51"/>
-      <c r="E25" s="51"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="56"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="78"/>
-      <c r="J25" s="80"/>
-      <c r="K25" s="56"/>
-      <c r="L25" s="56"/>
-      <c r="M25" s="70"/>
-      <c r="N25" s="82"/>
-      <c r="O25" s="55"/>
-      <c r="P25" s="92"/>
-      <c r="Q25" s="96"/>
-    </row>
-    <row r="26" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="72"/>
-      <c r="B26" s="60"/>
-      <c r="C26" s="58"/>
-      <c r="D26" s="51"/>
-      <c r="E26" s="51"/>
-      <c r="F26" s="56"/>
-      <c r="G26" s="56"/>
-      <c r="H26" s="56"/>
-      <c r="I26" s="78"/>
-      <c r="J26" s="80"/>
-      <c r="K26" s="56"/>
-      <c r="L26" s="56"/>
-      <c r="M26" s="70"/>
-      <c r="N26" s="82"/>
-      <c r="O26" s="55"/>
-      <c r="P26" s="92"/>
-      <c r="Q26" s="96"/>
-    </row>
-    <row r="27" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="72"/>
-      <c r="B27" s="60"/>
-      <c r="C27" s="59"/>
-      <c r="D27" s="51"/>
-      <c r="E27" s="51"/>
-      <c r="F27" s="56"/>
-      <c r="G27" s="56"/>
-      <c r="H27" s="56"/>
-      <c r="I27" s="78"/>
-      <c r="J27" s="80"/>
-      <c r="K27" s="56"/>
-      <c r="L27" s="56"/>
-      <c r="M27" s="66">
-        <v>2025</v>
-      </c>
-      <c r="N27" s="79"/>
-      <c r="O27" s="66"/>
-      <c r="P27" s="92"/>
-      <c r="Q27" s="96"/>
-    </row>
-    <row r="28" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="95"/>
-      <c r="B28" s="48"/>
-      <c r="C28" s="49"/>
-      <c r="D28" s="51"/>
-      <c r="E28" s="51"/>
-      <c r="F28" s="56"/>
-      <c r="G28" s="56"/>
-      <c r="H28" s="56"/>
-      <c r="I28" s="78"/>
-      <c r="J28" s="80"/>
-      <c r="K28" s="56"/>
-      <c r="L28" s="56"/>
-      <c r="M28" s="56"/>
-      <c r="N28" s="78"/>
-      <c r="O28" s="55"/>
-      <c r="P28" s="92"/>
-      <c r="Q28" s="96"/>
-    </row>
-    <row r="29" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="99"/>
-      <c r="B29" s="62"/>
-      <c r="C29" s="68"/>
-      <c r="D29" s="76"/>
-      <c r="E29" s="76"/>
-      <c r="F29" s="63"/>
-      <c r="G29" s="63"/>
-      <c r="H29" s="63"/>
-      <c r="I29" s="81"/>
-      <c r="J29" s="89"/>
-      <c r="K29" s="63"/>
-      <c r="L29" s="63"/>
-      <c r="M29" s="63"/>
-      <c r="N29" s="81"/>
-      <c r="O29" s="62"/>
-      <c r="P29" s="94"/>
-      <c r="Q29" s="100"/>
+    <row r="9" spans="1:17" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="76"/>
+      <c r="B9" s="77" t="s">
+        <v>168</v>
+      </c>
+      <c r="C9" s="78"/>
+      <c r="D9" s="82" t="s">
+        <v>169</v>
+      </c>
+      <c r="E9" s="82" t="s">
+        <v>170</v>
+      </c>
+      <c r="F9" s="83">
+        <v>46310</v>
+      </c>
+      <c r="G9" s="83"/>
+      <c r="H9" s="83"/>
+      <c r="I9" s="79"/>
+      <c r="J9" s="84"/>
+      <c r="K9" s="83"/>
+      <c r="L9" s="83"/>
+      <c r="M9" s="83"/>
+      <c r="N9" s="80"/>
+      <c r="O9" s="81">
+        <v>1</v>
+      </c>
+      <c r="P9" s="85"/>
+      <c r="Q9" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4718,31 +4072,10 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="B4">
-    <cfRule type="duplicateValues" dxfId="10" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B16">
-    <cfRule type="duplicateValues" dxfId="9" priority="133"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B18 B6:B14">
-    <cfRule type="duplicateValues" dxfId="8" priority="20161"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B20">
-    <cfRule type="duplicateValues" dxfId="7" priority="1129"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B21">
-    <cfRule type="duplicateValues" dxfId="6" priority="2971"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B22 B19">
-    <cfRule type="duplicateValues" dxfId="5" priority="16129"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B23:B26">
-    <cfRule type="duplicateValues" dxfId="4" priority="20773"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B27">
-    <cfRule type="duplicateValues" dxfId="3" priority="5676"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B28">
-    <cfRule type="duplicateValues" dxfId="2" priority="1811"/>
+  <conditionalFormatting sqref="B6:B9">
+    <cfRule type="duplicateValues" dxfId="2" priority="20777"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -4836,7 +4169,7 @@
     <row r="1" spans="1:69" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:69" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="46" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C2" s="47">
         <v>27</v>
@@ -4844,315 +4177,315 @@
     </row>
     <row r="3" spans="1:69" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="133" t="s">
+      <c r="A4" s="109" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="117"/>
+      <c r="C4" s="109" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="141"/>
-      <c r="C4" s="133" t="s">
+      <c r="D4" s="118"/>
+      <c r="E4" s="118"/>
+      <c r="F4" s="118"/>
+      <c r="G4" s="118"/>
+      <c r="H4" s="119"/>
+      <c r="I4" s="96" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="142"/>
-      <c r="E4" s="142"/>
-      <c r="F4" s="142"/>
-      <c r="G4" s="142"/>
-      <c r="H4" s="143"/>
-      <c r="I4" s="120" t="s">
+      <c r="J4" s="97"/>
+      <c r="K4" s="98"/>
+      <c r="L4" s="99"/>
+      <c r="M4" s="99"/>
+      <c r="N4" s="100"/>
+      <c r="O4" s="124" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="121"/>
-      <c r="K4" s="122"/>
-      <c r="L4" s="123"/>
-      <c r="M4" s="123"/>
-      <c r="N4" s="124"/>
-      <c r="O4" s="148" t="s">
+      <c r="P4" s="123" t="s">
         <v>24</v>
       </c>
-      <c r="P4" s="147" t="s">
+      <c r="Q4" s="124"/>
+      <c r="R4" s="124"/>
+      <c r="S4" s="124"/>
+      <c r="T4" s="124"/>
+      <c r="U4" s="125"/>
+      <c r="V4" s="106" t="s">
         <v>25</v>
       </c>
-      <c r="Q4" s="148"/>
-      <c r="R4" s="148"/>
-      <c r="S4" s="148"/>
-      <c r="T4" s="148"/>
-      <c r="U4" s="149"/>
-      <c r="V4" s="130" t="s">
-        <v>26</v>
-      </c>
-      <c r="W4" s="131"/>
-      <c r="X4" s="131"/>
-      <c r="Y4" s="131"/>
-      <c r="Z4" s="131"/>
-      <c r="AA4" s="131"/>
-      <c r="AB4" s="131"/>
-      <c r="AC4" s="131"/>
-      <c r="AD4" s="131"/>
-      <c r="AE4" s="131"/>
-      <c r="AF4" s="131"/>
-      <c r="AG4" s="131"/>
-      <c r="AH4" s="131"/>
-      <c r="AI4" s="131"/>
-      <c r="AJ4" s="131"/>
-      <c r="AK4" s="131"/>
-      <c r="AL4" s="131"/>
-      <c r="AM4" s="131"/>
-      <c r="AN4" s="131"/>
-      <c r="AO4" s="131"/>
-      <c r="AP4" s="131"/>
-      <c r="AQ4" s="131"/>
-      <c r="AR4" s="131"/>
-      <c r="AS4" s="131"/>
-      <c r="AT4" s="131"/>
-      <c r="AU4" s="131"/>
-      <c r="AV4" s="131"/>
-      <c r="AW4" s="131"/>
-      <c r="AX4" s="131"/>
-      <c r="AY4" s="131"/>
-      <c r="AZ4" s="131"/>
-      <c r="BA4" s="131"/>
-      <c r="BB4" s="131"/>
-      <c r="BC4" s="131"/>
-      <c r="BD4" s="131"/>
-      <c r="BE4" s="131"/>
-      <c r="BF4" s="131"/>
-      <c r="BG4" s="131"/>
-      <c r="BH4" s="131"/>
-      <c r="BI4" s="131"/>
-      <c r="BJ4" s="131"/>
-      <c r="BK4" s="131"/>
-      <c r="BL4" s="131"/>
-      <c r="BM4" s="131"/>
-      <c r="BN4" s="131"/>
-      <c r="BO4" s="131"/>
-      <c r="BP4" s="131"/>
-      <c r="BQ4" s="132"/>
+      <c r="W4" s="107"/>
+      <c r="X4" s="107"/>
+      <c r="Y4" s="107"/>
+      <c r="Z4" s="107"/>
+      <c r="AA4" s="107"/>
+      <c r="AB4" s="107"/>
+      <c r="AC4" s="107"/>
+      <c r="AD4" s="107"/>
+      <c r="AE4" s="107"/>
+      <c r="AF4" s="107"/>
+      <c r="AG4" s="107"/>
+      <c r="AH4" s="107"/>
+      <c r="AI4" s="107"/>
+      <c r="AJ4" s="107"/>
+      <c r="AK4" s="107"/>
+      <c r="AL4" s="107"/>
+      <c r="AM4" s="107"/>
+      <c r="AN4" s="107"/>
+      <c r="AO4" s="107"/>
+      <c r="AP4" s="107"/>
+      <c r="AQ4" s="107"/>
+      <c r="AR4" s="107"/>
+      <c r="AS4" s="107"/>
+      <c r="AT4" s="107"/>
+      <c r="AU4" s="107"/>
+      <c r="AV4" s="107"/>
+      <c r="AW4" s="107"/>
+      <c r="AX4" s="107"/>
+      <c r="AY4" s="107"/>
+      <c r="AZ4" s="107"/>
+      <c r="BA4" s="107"/>
+      <c r="BB4" s="107"/>
+      <c r="BC4" s="107"/>
+      <c r="BD4" s="107"/>
+      <c r="BE4" s="107"/>
+      <c r="BF4" s="107"/>
+      <c r="BG4" s="107"/>
+      <c r="BH4" s="107"/>
+      <c r="BI4" s="107"/>
+      <c r="BJ4" s="107"/>
+      <c r="BK4" s="107"/>
+      <c r="BL4" s="107"/>
+      <c r="BM4" s="107"/>
+      <c r="BN4" s="107"/>
+      <c r="BO4" s="107"/>
+      <c r="BP4" s="107"/>
+      <c r="BQ4" s="108"/>
     </row>
     <row r="5" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="134"/>
-      <c r="B5" s="141"/>
-      <c r="C5" s="144"/>
-      <c r="D5" s="145"/>
-      <c r="E5" s="145"/>
-      <c r="F5" s="145"/>
-      <c r="G5" s="145"/>
-      <c r="H5" s="146"/>
-      <c r="I5" s="125"/>
-      <c r="J5" s="126"/>
-      <c r="K5" s="127"/>
-      <c r="L5" s="128"/>
-      <c r="M5" s="128"/>
-      <c r="N5" s="129"/>
-      <c r="O5" s="153"/>
-      <c r="P5" s="150"/>
-      <c r="Q5" s="151"/>
-      <c r="R5" s="151"/>
-      <c r="S5" s="151"/>
-      <c r="T5" s="151"/>
-      <c r="U5" s="152"/>
-      <c r="V5" s="135" t="s">
+      <c r="A5" s="110"/>
+      <c r="B5" s="117"/>
+      <c r="C5" s="120"/>
+      <c r="D5" s="121"/>
+      <c r="E5" s="121"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="121"/>
+      <c r="H5" s="122"/>
+      <c r="I5" s="101"/>
+      <c r="J5" s="102"/>
+      <c r="K5" s="103"/>
+      <c r="L5" s="104"/>
+      <c r="M5" s="104"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="129"/>
+      <c r="P5" s="126"/>
+      <c r="Q5" s="127"/>
+      <c r="R5" s="127"/>
+      <c r="S5" s="127"/>
+      <c r="T5" s="127"/>
+      <c r="U5" s="128"/>
+      <c r="V5" s="111" t="s">
         <v>19</v>
       </c>
-      <c r="W5" s="136"/>
-      <c r="X5" s="136"/>
-      <c r="Y5" s="136"/>
-      <c r="Z5" s="136"/>
-      <c r="AA5" s="137"/>
-      <c r="AB5" s="138" t="s">
+      <c r="W5" s="112"/>
+      <c r="X5" s="112"/>
+      <c r="Y5" s="112"/>
+      <c r="Z5" s="112"/>
+      <c r="AA5" s="113"/>
+      <c r="AB5" s="114" t="s">
         <v>18</v>
       </c>
-      <c r="AC5" s="139"/>
-      <c r="AD5" s="139"/>
-      <c r="AE5" s="139"/>
-      <c r="AF5" s="139"/>
-      <c r="AG5" s="140"/>
-      <c r="AH5" s="138" t="s">
+      <c r="AC5" s="115"/>
+      <c r="AD5" s="115"/>
+      <c r="AE5" s="115"/>
+      <c r="AF5" s="115"/>
+      <c r="AG5" s="116"/>
+      <c r="AH5" s="114" t="s">
+        <v>26</v>
+      </c>
+      <c r="AI5" s="115"/>
+      <c r="AJ5" s="115"/>
+      <c r="AK5" s="115"/>
+      <c r="AL5" s="115"/>
+      <c r="AM5" s="116"/>
+      <c r="AN5" s="114" t="s">
         <v>27</v>
       </c>
-      <c r="AI5" s="139"/>
-      <c r="AJ5" s="139"/>
-      <c r="AK5" s="139"/>
-      <c r="AL5" s="139"/>
-      <c r="AM5" s="140"/>
-      <c r="AN5" s="138" t="s">
+      <c r="AO5" s="115"/>
+      <c r="AP5" s="115"/>
+      <c r="AQ5" s="115"/>
+      <c r="AR5" s="115"/>
+      <c r="AS5" s="116"/>
+      <c r="AT5" s="114" t="s">
         <v>28</v>
       </c>
-      <c r="AO5" s="139"/>
-      <c r="AP5" s="139"/>
-      <c r="AQ5" s="139"/>
-      <c r="AR5" s="139"/>
-      <c r="AS5" s="140"/>
-      <c r="AT5" s="138" t="s">
+      <c r="AU5" s="115"/>
+      <c r="AV5" s="115"/>
+      <c r="AW5" s="115"/>
+      <c r="AX5" s="115"/>
+      <c r="AY5" s="116"/>
+      <c r="AZ5" s="114" t="s">
         <v>29</v>
       </c>
-      <c r="AU5" s="139"/>
-      <c r="AV5" s="139"/>
-      <c r="AW5" s="139"/>
-      <c r="AX5" s="139"/>
-      <c r="AY5" s="140"/>
-      <c r="AZ5" s="138" t="s">
+      <c r="BA5" s="115"/>
+      <c r="BB5" s="115"/>
+      <c r="BC5" s="115"/>
+      <c r="BD5" s="115"/>
+      <c r="BE5" s="116"/>
+      <c r="BF5" s="114" t="s">
         <v>30</v>
       </c>
-      <c r="BA5" s="139"/>
-      <c r="BB5" s="139"/>
-      <c r="BC5" s="139"/>
-      <c r="BD5" s="139"/>
-      <c r="BE5" s="140"/>
-      <c r="BF5" s="138" t="s">
+      <c r="BG5" s="115"/>
+      <c r="BH5" s="115"/>
+      <c r="BI5" s="115"/>
+      <c r="BJ5" s="115"/>
+      <c r="BK5" s="116"/>
+      <c r="BL5" s="96" t="s">
         <v>31</v>
       </c>
-      <c r="BG5" s="139"/>
-      <c r="BH5" s="139"/>
-      <c r="BI5" s="139"/>
-      <c r="BJ5" s="139"/>
-      <c r="BK5" s="140"/>
-      <c r="BL5" s="120" t="s">
-        <v>32</v>
-      </c>
-      <c r="BM5" s="122"/>
-      <c r="BN5" s="122"/>
-      <c r="BO5" s="123"/>
-      <c r="BP5" s="123"/>
-      <c r="BQ5" s="124"/>
+      <c r="BM5" s="98"/>
+      <c r="BN5" s="98"/>
+      <c r="BO5" s="99"/>
+      <c r="BP5" s="99"/>
+      <c r="BQ5" s="100"/>
     </row>
     <row r="6" spans="1:69" ht="103.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="134"/>
-      <c r="B6" s="119"/>
-      <c r="C6" s="114" t="s">
+      <c r="A6" s="110"/>
+      <c r="B6" s="95"/>
+      <c r="C6" s="90" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="91"/>
+      <c r="E6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="115"/>
-      <c r="E6" s="114" t="s">
+      <c r="F6" s="91"/>
+      <c r="G6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="115"/>
-      <c r="G6" s="114" t="s">
-        <v>35</v>
-      </c>
-      <c r="H6" s="115"/>
-      <c r="I6" s="114" t="s">
+      <c r="H6" s="91"/>
+      <c r="I6" s="90" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6" s="91"/>
+      <c r="K6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="J6" s="115"/>
-      <c r="K6" s="114" t="s">
+      <c r="L6" s="91"/>
+      <c r="M6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="115"/>
-      <c r="M6" s="114" t="s">
-        <v>35</v>
-      </c>
-      <c r="N6" s="115"/>
-      <c r="O6" s="151"/>
-      <c r="P6" s="114" t="s">
+      <c r="N6" s="91"/>
+      <c r="O6" s="127"/>
+      <c r="P6" s="90" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q6" s="91"/>
+      <c r="R6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="Q6" s="115"/>
-      <c r="R6" s="114" t="s">
+      <c r="S6" s="91"/>
+      <c r="T6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="S6" s="115"/>
-      <c r="T6" s="114" t="s">
-        <v>35</v>
-      </c>
-      <c r="U6" s="115"/>
-      <c r="V6" s="119" t="s">
+      <c r="U6" s="91"/>
+      <c r="V6" s="95" t="s">
+        <v>32</v>
+      </c>
+      <c r="W6" s="94"/>
+      <c r="X6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="W6" s="118"/>
-      <c r="X6" s="116" t="s">
+      <c r="Y6" s="94"/>
+      <c r="Z6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="Y6" s="118"/>
-      <c r="Z6" s="116" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA6" s="117"/>
-      <c r="AB6" s="119" t="s">
+      <c r="AA6" s="93"/>
+      <c r="AB6" s="95" t="s">
+        <v>32</v>
+      </c>
+      <c r="AC6" s="94"/>
+      <c r="AD6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AC6" s="118"/>
-      <c r="AD6" s="116" t="s">
+      <c r="AE6" s="94"/>
+      <c r="AF6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AE6" s="118"/>
-      <c r="AF6" s="116" t="s">
-        <v>35</v>
-      </c>
-      <c r="AG6" s="117"/>
-      <c r="AH6" s="119" t="s">
+      <c r="AG6" s="93"/>
+      <c r="AH6" s="95" t="s">
+        <v>32</v>
+      </c>
+      <c r="AI6" s="94"/>
+      <c r="AJ6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AI6" s="118"/>
-      <c r="AJ6" s="116" t="s">
+      <c r="AK6" s="94"/>
+      <c r="AL6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AK6" s="118"/>
-      <c r="AL6" s="116" t="s">
-        <v>35</v>
-      </c>
-      <c r="AM6" s="117"/>
-      <c r="AN6" s="119" t="s">
+      <c r="AM6" s="93"/>
+      <c r="AN6" s="95" t="s">
+        <v>32</v>
+      </c>
+      <c r="AO6" s="94"/>
+      <c r="AP6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AO6" s="118"/>
-      <c r="AP6" s="116" t="s">
+      <c r="AQ6" s="94"/>
+      <c r="AR6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AQ6" s="118"/>
-      <c r="AR6" s="116" t="s">
-        <v>35</v>
-      </c>
-      <c r="AS6" s="117"/>
-      <c r="AT6" s="119" t="s">
+      <c r="AS6" s="93"/>
+      <c r="AT6" s="95" t="s">
+        <v>32</v>
+      </c>
+      <c r="AU6" s="94"/>
+      <c r="AV6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AU6" s="118"/>
-      <c r="AV6" s="116" t="s">
+      <c r="AW6" s="94"/>
+      <c r="AX6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AW6" s="118"/>
-      <c r="AX6" s="116" t="s">
-        <v>35</v>
-      </c>
-      <c r="AY6" s="117"/>
-      <c r="AZ6" s="119" t="s">
+      <c r="AY6" s="93"/>
+      <c r="AZ6" s="95" t="s">
+        <v>32</v>
+      </c>
+      <c r="BA6" s="94"/>
+      <c r="BB6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BA6" s="118"/>
-      <c r="BB6" s="116" t="s">
+      <c r="BC6" s="94"/>
+      <c r="BD6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BC6" s="118"/>
-      <c r="BD6" s="116" t="s">
-        <v>35</v>
-      </c>
-      <c r="BE6" s="117"/>
-      <c r="BF6" s="119" t="s">
+      <c r="BE6" s="93"/>
+      <c r="BF6" s="95" t="s">
+        <v>32</v>
+      </c>
+      <c r="BG6" s="94"/>
+      <c r="BH6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BG6" s="118"/>
-      <c r="BH6" s="116" t="s">
+      <c r="BI6" s="94"/>
+      <c r="BJ6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BI6" s="118"/>
-      <c r="BJ6" s="116" t="s">
-        <v>35</v>
-      </c>
-      <c r="BK6" s="117"/>
-      <c r="BL6" s="119" t="s">
+      <c r="BK6" s="93"/>
+      <c r="BL6" s="95" t="s">
+        <v>32</v>
+      </c>
+      <c r="BM6" s="94"/>
+      <c r="BN6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BM6" s="118"/>
-      <c r="BN6" s="116" t="s">
+      <c r="BO6" s="94"/>
+      <c r="BP6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BO6" s="118"/>
-      <c r="BP6" s="116" t="s">
-        <v>35</v>
-      </c>
-      <c r="BQ6" s="117"/>
+      <c r="BQ6" s="93"/>
     </row>
     <row r="7" spans="1:69" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B7" s="17">
         <f ca="1">IF(C2="",TEXT(TODAY(),"D"),C2)</f>
@@ -5178,27 +4511,27 @@
       <c r="T7" s="7"/>
       <c r="U7" s="26"/>
       <c r="V7" s="29" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="W7" s="23"/>
       <c r="X7" s="19" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="Y7" s="23"/>
       <c r="Z7" s="8"/>
       <c r="AA7" s="26"/>
       <c r="AB7" s="29" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="AC7" s="23"/>
       <c r="AD7" s="19" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="AE7" s="23"/>
       <c r="AF7" s="8"/>
       <c r="AG7" s="26"/>
       <c r="AH7" s="29" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="AI7" s="23"/>
       <c r="AJ7" s="8"/>
@@ -5206,7 +4539,7 @@
       <c r="AL7" s="8"/>
       <c r="AM7" s="26"/>
       <c r="AN7" s="29" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="AO7" s="23"/>
       <c r="AP7" s="8"/>
@@ -5214,17 +4547,17 @@
       <c r="AR7" s="8"/>
       <c r="AS7" s="26"/>
       <c r="AT7" s="29" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="AU7" s="23"/>
       <c r="AV7" s="19" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="AW7" s="23"/>
       <c r="AX7" s="8"/>
       <c r="AY7" s="26"/>
       <c r="AZ7" s="29" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="BA7" s="23"/>
       <c r="BB7" s="8"/>
@@ -5232,7 +4565,7 @@
       <c r="BD7" s="8"/>
       <c r="BE7" s="26"/>
       <c r="BF7" s="29" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="BG7" s="23"/>
       <c r="BH7" s="8"/>
@@ -5248,7 +4581,7 @@
     </row>
     <row r="8" spans="1:69" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="6" t="e">
@@ -5525,7 +4858,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C9" s="12" t="e">
         <f ca="1">COUNTIFS(INDIRECT($B9&amp;"["&amp;$B$7&amp;"]"),"&lt;&gt;",INDIRECT($B9&amp;"[ШПК]"),"&lt;&gt;",INDIRECT($B9&amp;"[ПІБ]"),"&lt;&gt;")-SUM(E9,G9)</f>
@@ -5798,10 +5131,10 @@
     </row>
     <row r="10" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C10" s="12" t="e">
         <f t="shared" ref="C10:C28" ca="1" si="20">COUNTIFS(INDIRECT($B10&amp;"["&amp;$B$7&amp;"]"),"&lt;&gt;",INDIRECT($B10&amp;"[ШПК]"),"&lt;&gt;",INDIRECT($B10&amp;"[ПІБ]"),"&lt;&gt;")-SUM(E10,G10)</f>
@@ -6074,10 +5407,10 @@
     </row>
     <row r="11" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C11" s="12" t="e">
         <f ca="1">COUNTIFS(INDIRECT($B11&amp;"["&amp;$B$7&amp;"]"),"&lt;&gt;",INDIRECT($B11&amp;"[ШПК]"),"&lt;&gt;",INDIRECT($B11&amp;"[ПІБ]"),"&lt;&gt;")-SUM(E11,G11)</f>
@@ -6350,10 +5683,10 @@
     </row>
     <row r="12" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B12" s="24" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C12" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -6626,10 +5959,10 @@
     </row>
     <row r="13" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C13" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -6902,10 +6235,10 @@
     </row>
     <row r="14" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C14" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -7178,10 +6511,10 @@
     </row>
     <row r="15" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C15" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -7454,10 +6787,10 @@
     </row>
     <row r="16" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C16" s="9" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -7730,10 +7063,10 @@
     </row>
     <row r="17" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C17" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -8006,10 +7339,10 @@
     </row>
     <row r="18" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C18" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -8282,10 +7615,10 @@
     </row>
     <row r="19" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C19" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -8558,10 +7891,10 @@
     </row>
     <row r="20" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C20" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -8834,10 +8167,10 @@
     </row>
     <row r="21" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B21" s="24" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C21" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -9110,10 +8443,10 @@
     </row>
     <row r="22" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B22" s="24" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C22" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -9386,10 +8719,10 @@
     </row>
     <row r="23" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B23" s="24" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C23" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -9662,10 +8995,10 @@
     </row>
     <row r="24" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B24" s="24" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C24" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -9938,10 +9271,10 @@
     </row>
     <row r="25" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C25" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -10214,10 +9547,10 @@
     </row>
     <row r="26" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B26" s="24" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C26" s="12" t="e">
         <f ca="1">COUNTIFS(INDIRECT($B26&amp;"["&amp;$B$7&amp;"]"),"&lt;&gt;",INDIRECT($B26&amp;"[ШПК]"),"&lt;&gt;",INDIRECT($B26&amp;"[ПІБ]"),"&lt;&gt;")-SUM(E26,G26)</f>
@@ -10490,10 +9823,10 @@
     </row>
     <row r="27" spans="1:69" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B27" s="24" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C27" s="12" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -10766,10 +10099,10 @@
     </row>
     <row r="28" spans="1:69" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="31" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B28" s="32" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C28" s="33" t="e">
         <f t="shared" ca="1" si="20"/>
@@ -11042,10 +10375,10 @@
     </row>
     <row r="29" spans="1:69" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="44" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B29" s="38" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C29" s="39" t="e">
         <f ca="1">COUNTIFS(INDIRECT($B29&amp;"["&amp;$B$7&amp;"]"),"&lt;&gt;",INDIRECT($B29&amp;"[ШПК]"),"&lt;&gt;",INDIRECT($B29&amp;"[ПІБ]"),"&lt;&gt;")-SUM(E29,G29)</f>
@@ -11298,31 +10631,31 @@
   <sheetData>
     <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>7</v>
@@ -11330,322 +10663,322 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="F2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="I2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="F3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="I3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="F4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="I4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="H7" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="K7" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>4</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>4</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="E9" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="H9" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J9" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="K9" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="E10" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G10" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="H10" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="K10" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F11" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="H11" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I11" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="J11" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="J11" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="K11" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -11656,124 +10989,124 @@
         <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>67</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F13" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>67</v>
-      </c>
       <c r="H13" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I13" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J13" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="J13" s="1" t="s">
-        <v>67</v>
-      </c>
       <c r="K13" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="E14" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F14" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="G14" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="H14" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I14" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="J14" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="K14" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="E15" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="H15" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="J15" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="J15" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="K15" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -11784,124 +11117,124 @@
         <v>6</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>6</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>6</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -11909,671 +11242,671 @@
         <v>6</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="D37" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -12581,31 +11914,31 @@
         <v>9</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -12613,36 +11946,36 @@
         <v>10</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
@@ -12657,112 +11990,112 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tmp: Align test milestones with completed operations and save test workbooks
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
+++ b/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\tests\PersonalEventBuilder\Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{570194B4-5804-4A7E-A871-96F650668B92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0CD8999-E563-470D-95FA-419E8AD74081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -633,10 +633,10 @@
     <t>БОНДАРЕНКО Олександр Юрійович</t>
   </si>
   <si>
-    <t>Щорічна відпустка</t>
-  </si>
-  <si>
     <t>м. Тестоград</t>
+  </si>
+  <si>
+    <t>Відпустка для лікування</t>
   </si>
 </sst>
 </file>
@@ -2268,125 +2268,125 @@
     <xf numFmtId="164" fontId="38" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="161">
@@ -4034,17 +4034,17 @@
       <c r="P8" s="65"/>
       <c r="Q8" s="56"/>
     </row>
-    <row r="9" spans="1:17" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A9" s="76"/>
       <c r="B9" s="77" t="s">
         <v>168</v>
       </c>
       <c r="C9" s="78"/>
       <c r="D9" s="82" t="s">
+        <v>170</v>
+      </c>
+      <c r="E9" s="82" t="s">
         <v>169</v>
-      </c>
-      <c r="E9" s="82" t="s">
-        <v>170</v>
       </c>
       <c r="F9" s="83">
         <v>46310</v>
@@ -4075,7 +4075,7 @@
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B9">
-    <cfRule type="duplicateValues" dxfId="2" priority="20777"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="20781"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -4177,311 +4177,311 @@
     </row>
     <row r="3" spans="1:69" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="109" t="s">
+      <c r="A4" s="103" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="117"/>
-      <c r="C4" s="109" t="s">
+      <c r="B4" s="111"/>
+      <c r="C4" s="103" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="118"/>
-      <c r="E4" s="118"/>
-      <c r="F4" s="118"/>
-      <c r="G4" s="118"/>
-      <c r="H4" s="119"/>
-      <c r="I4" s="96" t="s">
+      <c r="D4" s="115"/>
+      <c r="E4" s="115"/>
+      <c r="F4" s="115"/>
+      <c r="G4" s="115"/>
+      <c r="H4" s="116"/>
+      <c r="I4" s="90" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="97"/>
-      <c r="K4" s="98"/>
-      <c r="L4" s="99"/>
-      <c r="M4" s="99"/>
-      <c r="N4" s="100"/>
-      <c r="O4" s="124" t="s">
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
+      <c r="L4" s="93"/>
+      <c r="M4" s="93"/>
+      <c r="N4" s="94"/>
+      <c r="O4" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="P4" s="123" t="s">
+      <c r="P4" s="120" t="s">
         <v>24</v>
       </c>
-      <c r="Q4" s="124"/>
-      <c r="R4" s="124"/>
-      <c r="S4" s="124"/>
-      <c r="T4" s="124"/>
-      <c r="U4" s="125"/>
-      <c r="V4" s="106" t="s">
+      <c r="Q4" s="121"/>
+      <c r="R4" s="121"/>
+      <c r="S4" s="121"/>
+      <c r="T4" s="121"/>
+      <c r="U4" s="122"/>
+      <c r="V4" s="100" t="s">
         <v>25</v>
       </c>
-      <c r="W4" s="107"/>
-      <c r="X4" s="107"/>
-      <c r="Y4" s="107"/>
-      <c r="Z4" s="107"/>
-      <c r="AA4" s="107"/>
-      <c r="AB4" s="107"/>
-      <c r="AC4" s="107"/>
-      <c r="AD4" s="107"/>
-      <c r="AE4" s="107"/>
-      <c r="AF4" s="107"/>
-      <c r="AG4" s="107"/>
-      <c r="AH4" s="107"/>
-      <c r="AI4" s="107"/>
-      <c r="AJ4" s="107"/>
-      <c r="AK4" s="107"/>
-      <c r="AL4" s="107"/>
-      <c r="AM4" s="107"/>
-      <c r="AN4" s="107"/>
-      <c r="AO4" s="107"/>
-      <c r="AP4" s="107"/>
-      <c r="AQ4" s="107"/>
-      <c r="AR4" s="107"/>
-      <c r="AS4" s="107"/>
-      <c r="AT4" s="107"/>
-      <c r="AU4" s="107"/>
-      <c r="AV4" s="107"/>
-      <c r="AW4" s="107"/>
-      <c r="AX4" s="107"/>
-      <c r="AY4" s="107"/>
-      <c r="AZ4" s="107"/>
-      <c r="BA4" s="107"/>
-      <c r="BB4" s="107"/>
-      <c r="BC4" s="107"/>
-      <c r="BD4" s="107"/>
-      <c r="BE4" s="107"/>
-      <c r="BF4" s="107"/>
-      <c r="BG4" s="107"/>
-      <c r="BH4" s="107"/>
-      <c r="BI4" s="107"/>
-      <c r="BJ4" s="107"/>
-      <c r="BK4" s="107"/>
-      <c r="BL4" s="107"/>
-      <c r="BM4" s="107"/>
-      <c r="BN4" s="107"/>
-      <c r="BO4" s="107"/>
-      <c r="BP4" s="107"/>
-      <c r="BQ4" s="108"/>
+      <c r="W4" s="101"/>
+      <c r="X4" s="101"/>
+      <c r="Y4" s="101"/>
+      <c r="Z4" s="101"/>
+      <c r="AA4" s="101"/>
+      <c r="AB4" s="101"/>
+      <c r="AC4" s="101"/>
+      <c r="AD4" s="101"/>
+      <c r="AE4" s="101"/>
+      <c r="AF4" s="101"/>
+      <c r="AG4" s="101"/>
+      <c r="AH4" s="101"/>
+      <c r="AI4" s="101"/>
+      <c r="AJ4" s="101"/>
+      <c r="AK4" s="101"/>
+      <c r="AL4" s="101"/>
+      <c r="AM4" s="101"/>
+      <c r="AN4" s="101"/>
+      <c r="AO4" s="101"/>
+      <c r="AP4" s="101"/>
+      <c r="AQ4" s="101"/>
+      <c r="AR4" s="101"/>
+      <c r="AS4" s="101"/>
+      <c r="AT4" s="101"/>
+      <c r="AU4" s="101"/>
+      <c r="AV4" s="101"/>
+      <c r="AW4" s="101"/>
+      <c r="AX4" s="101"/>
+      <c r="AY4" s="101"/>
+      <c r="AZ4" s="101"/>
+      <c r="BA4" s="101"/>
+      <c r="BB4" s="101"/>
+      <c r="BC4" s="101"/>
+      <c r="BD4" s="101"/>
+      <c r="BE4" s="101"/>
+      <c r="BF4" s="101"/>
+      <c r="BG4" s="101"/>
+      <c r="BH4" s="101"/>
+      <c r="BI4" s="101"/>
+      <c r="BJ4" s="101"/>
+      <c r="BK4" s="101"/>
+      <c r="BL4" s="101"/>
+      <c r="BM4" s="101"/>
+      <c r="BN4" s="101"/>
+      <c r="BO4" s="101"/>
+      <c r="BP4" s="101"/>
+      <c r="BQ4" s="102"/>
     </row>
     <row r="5" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="110"/>
-      <c r="B5" s="117"/>
-      <c r="C5" s="120"/>
-      <c r="D5" s="121"/>
-      <c r="E5" s="121"/>
-      <c r="F5" s="121"/>
-      <c r="G5" s="121"/>
-      <c r="H5" s="122"/>
-      <c r="I5" s="101"/>
-      <c r="J5" s="102"/>
-      <c r="K5" s="103"/>
-      <c r="L5" s="104"/>
-      <c r="M5" s="104"/>
-      <c r="N5" s="105"/>
-      <c r="O5" s="129"/>
-      <c r="P5" s="126"/>
-      <c r="Q5" s="127"/>
-      <c r="R5" s="127"/>
-      <c r="S5" s="127"/>
-      <c r="T5" s="127"/>
-      <c r="U5" s="128"/>
-      <c r="V5" s="111" t="s">
+      <c r="A5" s="104"/>
+      <c r="B5" s="111"/>
+      <c r="C5" s="117"/>
+      <c r="D5" s="118"/>
+      <c r="E5" s="118"/>
+      <c r="F5" s="118"/>
+      <c r="G5" s="118"/>
+      <c r="H5" s="119"/>
+      <c r="I5" s="95"/>
+      <c r="J5" s="96"/>
+      <c r="K5" s="97"/>
+      <c r="L5" s="98"/>
+      <c r="M5" s="98"/>
+      <c r="N5" s="99"/>
+      <c r="O5" s="126"/>
+      <c r="P5" s="123"/>
+      <c r="Q5" s="124"/>
+      <c r="R5" s="124"/>
+      <c r="S5" s="124"/>
+      <c r="T5" s="124"/>
+      <c r="U5" s="125"/>
+      <c r="V5" s="105" t="s">
         <v>19</v>
       </c>
-      <c r="W5" s="112"/>
-      <c r="X5" s="112"/>
-      <c r="Y5" s="112"/>
-      <c r="Z5" s="112"/>
-      <c r="AA5" s="113"/>
-      <c r="AB5" s="114" t="s">
+      <c r="W5" s="106"/>
+      <c r="X5" s="106"/>
+      <c r="Y5" s="106"/>
+      <c r="Z5" s="106"/>
+      <c r="AA5" s="107"/>
+      <c r="AB5" s="108" t="s">
         <v>18</v>
       </c>
-      <c r="AC5" s="115"/>
-      <c r="AD5" s="115"/>
-      <c r="AE5" s="115"/>
-      <c r="AF5" s="115"/>
-      <c r="AG5" s="116"/>
-      <c r="AH5" s="114" t="s">
+      <c r="AC5" s="109"/>
+      <c r="AD5" s="109"/>
+      <c r="AE5" s="109"/>
+      <c r="AF5" s="109"/>
+      <c r="AG5" s="110"/>
+      <c r="AH5" s="108" t="s">
         <v>26</v>
       </c>
-      <c r="AI5" s="115"/>
-      <c r="AJ5" s="115"/>
-      <c r="AK5" s="115"/>
-      <c r="AL5" s="115"/>
-      <c r="AM5" s="116"/>
-      <c r="AN5" s="114" t="s">
+      <c r="AI5" s="109"/>
+      <c r="AJ5" s="109"/>
+      <c r="AK5" s="109"/>
+      <c r="AL5" s="109"/>
+      <c r="AM5" s="110"/>
+      <c r="AN5" s="108" t="s">
         <v>27</v>
       </c>
-      <c r="AO5" s="115"/>
-      <c r="AP5" s="115"/>
-      <c r="AQ5" s="115"/>
-      <c r="AR5" s="115"/>
-      <c r="AS5" s="116"/>
-      <c r="AT5" s="114" t="s">
+      <c r="AO5" s="109"/>
+      <c r="AP5" s="109"/>
+      <c r="AQ5" s="109"/>
+      <c r="AR5" s="109"/>
+      <c r="AS5" s="110"/>
+      <c r="AT5" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="AU5" s="115"/>
-      <c r="AV5" s="115"/>
-      <c r="AW5" s="115"/>
-      <c r="AX5" s="115"/>
-      <c r="AY5" s="116"/>
-      <c r="AZ5" s="114" t="s">
+      <c r="AU5" s="109"/>
+      <c r="AV5" s="109"/>
+      <c r="AW5" s="109"/>
+      <c r="AX5" s="109"/>
+      <c r="AY5" s="110"/>
+      <c r="AZ5" s="108" t="s">
         <v>29</v>
       </c>
-      <c r="BA5" s="115"/>
-      <c r="BB5" s="115"/>
-      <c r="BC5" s="115"/>
-      <c r="BD5" s="115"/>
-      <c r="BE5" s="116"/>
-      <c r="BF5" s="114" t="s">
+      <c r="BA5" s="109"/>
+      <c r="BB5" s="109"/>
+      <c r="BC5" s="109"/>
+      <c r="BD5" s="109"/>
+      <c r="BE5" s="110"/>
+      <c r="BF5" s="108" t="s">
         <v>30</v>
       </c>
-      <c r="BG5" s="115"/>
-      <c r="BH5" s="115"/>
-      <c r="BI5" s="115"/>
-      <c r="BJ5" s="115"/>
-      <c r="BK5" s="116"/>
-      <c r="BL5" s="96" t="s">
+      <c r="BG5" s="109"/>
+      <c r="BH5" s="109"/>
+      <c r="BI5" s="109"/>
+      <c r="BJ5" s="109"/>
+      <c r="BK5" s="110"/>
+      <c r="BL5" s="90" t="s">
         <v>31</v>
       </c>
-      <c r="BM5" s="98"/>
-      <c r="BN5" s="98"/>
-      <c r="BO5" s="99"/>
-      <c r="BP5" s="99"/>
-      <c r="BQ5" s="100"/>
+      <c r="BM5" s="92"/>
+      <c r="BN5" s="92"/>
+      <c r="BO5" s="93"/>
+      <c r="BP5" s="93"/>
+      <c r="BQ5" s="94"/>
     </row>
     <row r="6" spans="1:69" ht="103.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="110"/>
-      <c r="B6" s="95"/>
-      <c r="C6" s="90" t="s">
+      <c r="A6" s="104"/>
+      <c r="B6" s="112"/>
+      <c r="C6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="91"/>
-      <c r="E6" s="90" t="s">
+      <c r="D6" s="129"/>
+      <c r="E6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="91"/>
-      <c r="G6" s="90" t="s">
+      <c r="F6" s="129"/>
+      <c r="G6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="91"/>
-      <c r="I6" s="90" t="s">
+      <c r="H6" s="129"/>
+      <c r="I6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="J6" s="91"/>
-      <c r="K6" s="90" t="s">
+      <c r="J6" s="129"/>
+      <c r="K6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="L6" s="91"/>
-      <c r="M6" s="90" t="s">
+      <c r="L6" s="129"/>
+      <c r="M6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="N6" s="91"/>
-      <c r="O6" s="127"/>
-      <c r="P6" s="90" t="s">
+      <c r="N6" s="129"/>
+      <c r="O6" s="124"/>
+      <c r="P6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="Q6" s="91"/>
-      <c r="R6" s="90" t="s">
+      <c r="Q6" s="129"/>
+      <c r="R6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="S6" s="91"/>
-      <c r="T6" s="90" t="s">
+      <c r="S6" s="129"/>
+      <c r="T6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="U6" s="91"/>
-      <c r="V6" s="95" t="s">
+      <c r="U6" s="129"/>
+      <c r="V6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="W6" s="94"/>
-      <c r="X6" s="92" t="s">
+      <c r="W6" s="127"/>
+      <c r="X6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="Y6" s="94"/>
-      <c r="Z6" s="92" t="s">
+      <c r="Y6" s="127"/>
+      <c r="Z6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AA6" s="93"/>
-      <c r="AB6" s="95" t="s">
+      <c r="AA6" s="114"/>
+      <c r="AB6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AC6" s="94"/>
-      <c r="AD6" s="92" t="s">
+      <c r="AC6" s="127"/>
+      <c r="AD6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AE6" s="94"/>
-      <c r="AF6" s="92" t="s">
+      <c r="AE6" s="127"/>
+      <c r="AF6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AG6" s="93"/>
-      <c r="AH6" s="95" t="s">
+      <c r="AG6" s="114"/>
+      <c r="AH6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AI6" s="94"/>
-      <c r="AJ6" s="92" t="s">
+      <c r="AI6" s="127"/>
+      <c r="AJ6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AK6" s="94"/>
-      <c r="AL6" s="92" t="s">
+      <c r="AK6" s="127"/>
+      <c r="AL6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AM6" s="93"/>
-      <c r="AN6" s="95" t="s">
+      <c r="AM6" s="114"/>
+      <c r="AN6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AO6" s="94"/>
-      <c r="AP6" s="92" t="s">
+      <c r="AO6" s="127"/>
+      <c r="AP6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AQ6" s="94"/>
-      <c r="AR6" s="92" t="s">
+      <c r="AQ6" s="127"/>
+      <c r="AR6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AS6" s="93"/>
-      <c r="AT6" s="95" t="s">
+      <c r="AS6" s="114"/>
+      <c r="AT6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AU6" s="94"/>
-      <c r="AV6" s="92" t="s">
+      <c r="AU6" s="127"/>
+      <c r="AV6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AW6" s="94"/>
-      <c r="AX6" s="92" t="s">
+      <c r="AW6" s="127"/>
+      <c r="AX6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AY6" s="93"/>
-      <c r="AZ6" s="95" t="s">
+      <c r="AY6" s="114"/>
+      <c r="AZ6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BA6" s="94"/>
-      <c r="BB6" s="92" t="s">
+      <c r="BA6" s="127"/>
+      <c r="BB6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BC6" s="94"/>
-      <c r="BD6" s="92" t="s">
+      <c r="BC6" s="127"/>
+      <c r="BD6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BE6" s="93"/>
-      <c r="BF6" s="95" t="s">
+      <c r="BE6" s="114"/>
+      <c r="BF6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BG6" s="94"/>
-      <c r="BH6" s="92" t="s">
+      <c r="BG6" s="127"/>
+      <c r="BH6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BI6" s="94"/>
-      <c r="BJ6" s="92" t="s">
+      <c r="BI6" s="127"/>
+      <c r="BJ6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BK6" s="93"/>
-      <c r="BL6" s="95" t="s">
+      <c r="BK6" s="114"/>
+      <c r="BL6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BM6" s="94"/>
-      <c r="BN6" s="92" t="s">
+      <c r="BM6" s="127"/>
+      <c r="BN6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BO6" s="94"/>
-      <c r="BP6" s="92" t="s">
+      <c r="BO6" s="127"/>
+      <c r="BP6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BQ6" s="93"/>
+      <c r="BQ6" s="114"/>
     </row>
     <row r="7" spans="1:69" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
@@ -10552,6 +10552,38 @@
     </row>
   </sheetData>
   <mergeCells count="48">
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="AJ6:AK6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AD6:AE6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AT6:AU6"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="AP6:AQ6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="BD6:BE6"/>
+    <mergeCell ref="BB6:BC6"/>
+    <mergeCell ref="AZ6:BA6"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AV6:AW6"/>
+    <mergeCell ref="BN6:BO6"/>
+    <mergeCell ref="BL6:BM6"/>
+    <mergeCell ref="BJ6:BK6"/>
+    <mergeCell ref="BH6:BI6"/>
+    <mergeCell ref="BF6:BG6"/>
     <mergeCell ref="I4:N5"/>
     <mergeCell ref="V4:BQ4"/>
     <mergeCell ref="A4:A6"/>
@@ -10568,38 +10600,6 @@
     <mergeCell ref="C4:H5"/>
     <mergeCell ref="P4:U5"/>
     <mergeCell ref="O4:O6"/>
-    <mergeCell ref="BN6:BO6"/>
-    <mergeCell ref="BL6:BM6"/>
-    <mergeCell ref="BJ6:BK6"/>
-    <mergeCell ref="BH6:BI6"/>
-    <mergeCell ref="BF6:BG6"/>
-    <mergeCell ref="BD6:BE6"/>
-    <mergeCell ref="BB6:BC6"/>
-    <mergeCell ref="AZ6:BA6"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AV6:AW6"/>
-    <mergeCell ref="AT6:AU6"/>
-    <mergeCell ref="AR6:AS6"/>
-    <mergeCell ref="AP6:AQ6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="AJ6:AK6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AD6:AE6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="X6:Y6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="R6:S6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="G6:H6"/>
   </mergeCells>
   <conditionalFormatting sqref="D1:D1048576 F1:F1048576 H1:H1048576 J1:J1048576 L1:L1048576 N1:N1048576 Q1:Q1048576 S1:S1048576 U1:U1048576 W1:W1048576 Y1:Y1048576 AA1:AA1048576 AC1:AC1048576 AE1:AE1048576 AG1:AG1048576 AI1:AI1048576 AK1:AK1048576 AM1:AM1048576 AO1:AO1048576 AQ1:AQ1048576 AS1:AS1048576 AU1:AU1048576 AW1:AW1048576 AY1:AY1048576 BA1:BA1048576 BC1:BC1048576 BE1:BE1048576 BG1:BG1048576 BI1:BI1048576 BK1:BK1048576 BM1:BM1048576 BO1:BO1048576 BQ1:BQ1048576">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">

</xml_diff>

<commit_message>
tmp: Render PEB test results and document previews from fixture data
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
+++ b/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\tests\PersonalEventBuilder\Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0CD8999-E563-470D-95FA-419E8AD74081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAE89B2B-98C1-463D-8A36-62BA6DB564C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -636,7 +636,7 @@
     <t>м. Тестоград</t>
   </si>
   <si>
-    <t>Відпустка для лікування</t>
+    <t>Щорічна відпустка</t>
   </si>
 </sst>
 </file>
@@ -2268,6 +2268,24 @@
     <xf numFmtId="164" fontId="38" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2334,15 +2352,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2378,15 +2387,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="161">
@@ -4034,7 +4034,7 @@
       <c r="P8" s="65"/>
       <c r="Q8" s="56"/>
     </row>
-    <row r="9" spans="1:17" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A9" s="76"/>
       <c r="B9" s="77" t="s">
         <v>168</v>
@@ -4075,7 +4075,7 @@
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B9">
-    <cfRule type="duplicateValues" dxfId="2" priority="20781"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="20782"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -4177,311 +4177,311 @@
     </row>
     <row r="3" spans="1:69" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="103" t="s">
+      <c r="A4" s="109" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="111"/>
-      <c r="C4" s="103" t="s">
+      <c r="B4" s="117"/>
+      <c r="C4" s="109" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="115"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="116"/>
-      <c r="I4" s="90" t="s">
+      <c r="D4" s="118"/>
+      <c r="E4" s="118"/>
+      <c r="F4" s="118"/>
+      <c r="G4" s="118"/>
+      <c r="H4" s="119"/>
+      <c r="I4" s="96" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
-      <c r="L4" s="93"/>
-      <c r="M4" s="93"/>
-      <c r="N4" s="94"/>
-      <c r="O4" s="121" t="s">
+      <c r="J4" s="97"/>
+      <c r="K4" s="98"/>
+      <c r="L4" s="99"/>
+      <c r="M4" s="99"/>
+      <c r="N4" s="100"/>
+      <c r="O4" s="124" t="s">
         <v>23</v>
       </c>
-      <c r="P4" s="120" t="s">
+      <c r="P4" s="123" t="s">
         <v>24</v>
       </c>
-      <c r="Q4" s="121"/>
-      <c r="R4" s="121"/>
-      <c r="S4" s="121"/>
-      <c r="T4" s="121"/>
-      <c r="U4" s="122"/>
-      <c r="V4" s="100" t="s">
+      <c r="Q4" s="124"/>
+      <c r="R4" s="124"/>
+      <c r="S4" s="124"/>
+      <c r="T4" s="124"/>
+      <c r="U4" s="125"/>
+      <c r="V4" s="106" t="s">
         <v>25</v>
       </c>
-      <c r="W4" s="101"/>
-      <c r="X4" s="101"/>
-      <c r="Y4" s="101"/>
-      <c r="Z4" s="101"/>
-      <c r="AA4" s="101"/>
-      <c r="AB4" s="101"/>
-      <c r="AC4" s="101"/>
-      <c r="AD4" s="101"/>
-      <c r="AE4" s="101"/>
-      <c r="AF4" s="101"/>
-      <c r="AG4" s="101"/>
-      <c r="AH4" s="101"/>
-      <c r="AI4" s="101"/>
-      <c r="AJ4" s="101"/>
-      <c r="AK4" s="101"/>
-      <c r="AL4" s="101"/>
-      <c r="AM4" s="101"/>
-      <c r="AN4" s="101"/>
-      <c r="AO4" s="101"/>
-      <c r="AP4" s="101"/>
-      <c r="AQ4" s="101"/>
-      <c r="AR4" s="101"/>
-      <c r="AS4" s="101"/>
-      <c r="AT4" s="101"/>
-      <c r="AU4" s="101"/>
-      <c r="AV4" s="101"/>
-      <c r="AW4" s="101"/>
-      <c r="AX4" s="101"/>
-      <c r="AY4" s="101"/>
-      <c r="AZ4" s="101"/>
-      <c r="BA4" s="101"/>
-      <c r="BB4" s="101"/>
-      <c r="BC4" s="101"/>
-      <c r="BD4" s="101"/>
-      <c r="BE4" s="101"/>
-      <c r="BF4" s="101"/>
-      <c r="BG4" s="101"/>
-      <c r="BH4" s="101"/>
-      <c r="BI4" s="101"/>
-      <c r="BJ4" s="101"/>
-      <c r="BK4" s="101"/>
-      <c r="BL4" s="101"/>
-      <c r="BM4" s="101"/>
-      <c r="BN4" s="101"/>
-      <c r="BO4" s="101"/>
-      <c r="BP4" s="101"/>
-      <c r="BQ4" s="102"/>
+      <c r="W4" s="107"/>
+      <c r="X4" s="107"/>
+      <c r="Y4" s="107"/>
+      <c r="Z4" s="107"/>
+      <c r="AA4" s="107"/>
+      <c r="AB4" s="107"/>
+      <c r="AC4" s="107"/>
+      <c r="AD4" s="107"/>
+      <c r="AE4" s="107"/>
+      <c r="AF4" s="107"/>
+      <c r="AG4" s="107"/>
+      <c r="AH4" s="107"/>
+      <c r="AI4" s="107"/>
+      <c r="AJ4" s="107"/>
+      <c r="AK4" s="107"/>
+      <c r="AL4" s="107"/>
+      <c r="AM4" s="107"/>
+      <c r="AN4" s="107"/>
+      <c r="AO4" s="107"/>
+      <c r="AP4" s="107"/>
+      <c r="AQ4" s="107"/>
+      <c r="AR4" s="107"/>
+      <c r="AS4" s="107"/>
+      <c r="AT4" s="107"/>
+      <c r="AU4" s="107"/>
+      <c r="AV4" s="107"/>
+      <c r="AW4" s="107"/>
+      <c r="AX4" s="107"/>
+      <c r="AY4" s="107"/>
+      <c r="AZ4" s="107"/>
+      <c r="BA4" s="107"/>
+      <c r="BB4" s="107"/>
+      <c r="BC4" s="107"/>
+      <c r="BD4" s="107"/>
+      <c r="BE4" s="107"/>
+      <c r="BF4" s="107"/>
+      <c r="BG4" s="107"/>
+      <c r="BH4" s="107"/>
+      <c r="BI4" s="107"/>
+      <c r="BJ4" s="107"/>
+      <c r="BK4" s="107"/>
+      <c r="BL4" s="107"/>
+      <c r="BM4" s="107"/>
+      <c r="BN4" s="107"/>
+      <c r="BO4" s="107"/>
+      <c r="BP4" s="107"/>
+      <c r="BQ4" s="108"/>
     </row>
     <row r="5" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="104"/>
-      <c r="B5" s="111"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="118"/>
-      <c r="E5" s="118"/>
-      <c r="F5" s="118"/>
-      <c r="G5" s="118"/>
-      <c r="H5" s="119"/>
-      <c r="I5" s="95"/>
-      <c r="J5" s="96"/>
-      <c r="K5" s="97"/>
-      <c r="L5" s="98"/>
-      <c r="M5" s="98"/>
-      <c r="N5" s="99"/>
-      <c r="O5" s="126"/>
-      <c r="P5" s="123"/>
-      <c r="Q5" s="124"/>
-      <c r="R5" s="124"/>
-      <c r="S5" s="124"/>
-      <c r="T5" s="124"/>
-      <c r="U5" s="125"/>
-      <c r="V5" s="105" t="s">
+      <c r="A5" s="110"/>
+      <c r="B5" s="117"/>
+      <c r="C5" s="120"/>
+      <c r="D5" s="121"/>
+      <c r="E5" s="121"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="121"/>
+      <c r="H5" s="122"/>
+      <c r="I5" s="101"/>
+      <c r="J5" s="102"/>
+      <c r="K5" s="103"/>
+      <c r="L5" s="104"/>
+      <c r="M5" s="104"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="129"/>
+      <c r="P5" s="126"/>
+      <c r="Q5" s="127"/>
+      <c r="R5" s="127"/>
+      <c r="S5" s="127"/>
+      <c r="T5" s="127"/>
+      <c r="U5" s="128"/>
+      <c r="V5" s="111" t="s">
         <v>19</v>
       </c>
-      <c r="W5" s="106"/>
-      <c r="X5" s="106"/>
-      <c r="Y5" s="106"/>
-      <c r="Z5" s="106"/>
-      <c r="AA5" s="107"/>
-      <c r="AB5" s="108" t="s">
+      <c r="W5" s="112"/>
+      <c r="X5" s="112"/>
+      <c r="Y5" s="112"/>
+      <c r="Z5" s="112"/>
+      <c r="AA5" s="113"/>
+      <c r="AB5" s="114" t="s">
         <v>18</v>
       </c>
-      <c r="AC5" s="109"/>
-      <c r="AD5" s="109"/>
-      <c r="AE5" s="109"/>
-      <c r="AF5" s="109"/>
-      <c r="AG5" s="110"/>
-      <c r="AH5" s="108" t="s">
+      <c r="AC5" s="115"/>
+      <c r="AD5" s="115"/>
+      <c r="AE5" s="115"/>
+      <c r="AF5" s="115"/>
+      <c r="AG5" s="116"/>
+      <c r="AH5" s="114" t="s">
         <v>26</v>
       </c>
-      <c r="AI5" s="109"/>
-      <c r="AJ5" s="109"/>
-      <c r="AK5" s="109"/>
-      <c r="AL5" s="109"/>
-      <c r="AM5" s="110"/>
-      <c r="AN5" s="108" t="s">
+      <c r="AI5" s="115"/>
+      <c r="AJ5" s="115"/>
+      <c r="AK5" s="115"/>
+      <c r="AL5" s="115"/>
+      <c r="AM5" s="116"/>
+      <c r="AN5" s="114" t="s">
         <v>27</v>
       </c>
-      <c r="AO5" s="109"/>
-      <c r="AP5" s="109"/>
-      <c r="AQ5" s="109"/>
-      <c r="AR5" s="109"/>
-      <c r="AS5" s="110"/>
-      <c r="AT5" s="108" t="s">
+      <c r="AO5" s="115"/>
+      <c r="AP5" s="115"/>
+      <c r="AQ5" s="115"/>
+      <c r="AR5" s="115"/>
+      <c r="AS5" s="116"/>
+      <c r="AT5" s="114" t="s">
         <v>28</v>
       </c>
-      <c r="AU5" s="109"/>
-      <c r="AV5" s="109"/>
-      <c r="AW5" s="109"/>
-      <c r="AX5" s="109"/>
-      <c r="AY5" s="110"/>
-      <c r="AZ5" s="108" t="s">
+      <c r="AU5" s="115"/>
+      <c r="AV5" s="115"/>
+      <c r="AW5" s="115"/>
+      <c r="AX5" s="115"/>
+      <c r="AY5" s="116"/>
+      <c r="AZ5" s="114" t="s">
         <v>29</v>
       </c>
-      <c r="BA5" s="109"/>
-      <c r="BB5" s="109"/>
-      <c r="BC5" s="109"/>
-      <c r="BD5" s="109"/>
-      <c r="BE5" s="110"/>
-      <c r="BF5" s="108" t="s">
+      <c r="BA5" s="115"/>
+      <c r="BB5" s="115"/>
+      <c r="BC5" s="115"/>
+      <c r="BD5" s="115"/>
+      <c r="BE5" s="116"/>
+      <c r="BF5" s="114" t="s">
         <v>30</v>
       </c>
-      <c r="BG5" s="109"/>
-      <c r="BH5" s="109"/>
-      <c r="BI5" s="109"/>
-      <c r="BJ5" s="109"/>
-      <c r="BK5" s="110"/>
-      <c r="BL5" s="90" t="s">
+      <c r="BG5" s="115"/>
+      <c r="BH5" s="115"/>
+      <c r="BI5" s="115"/>
+      <c r="BJ5" s="115"/>
+      <c r="BK5" s="116"/>
+      <c r="BL5" s="96" t="s">
         <v>31</v>
       </c>
-      <c r="BM5" s="92"/>
-      <c r="BN5" s="92"/>
-      <c r="BO5" s="93"/>
-      <c r="BP5" s="93"/>
-      <c r="BQ5" s="94"/>
+      <c r="BM5" s="98"/>
+      <c r="BN5" s="98"/>
+      <c r="BO5" s="99"/>
+      <c r="BP5" s="99"/>
+      <c r="BQ5" s="100"/>
     </row>
     <row r="6" spans="1:69" ht="103.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="104"/>
-      <c r="B6" s="112"/>
-      <c r="C6" s="128" t="s">
+      <c r="A6" s="110"/>
+      <c r="B6" s="95"/>
+      <c r="C6" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="129"/>
-      <c r="E6" s="128" t="s">
+      <c r="D6" s="91"/>
+      <c r="E6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="129"/>
-      <c r="G6" s="128" t="s">
+      <c r="F6" s="91"/>
+      <c r="G6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="129"/>
-      <c r="I6" s="128" t="s">
+      <c r="H6" s="91"/>
+      <c r="I6" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="J6" s="129"/>
-      <c r="K6" s="128" t="s">
+      <c r="J6" s="91"/>
+      <c r="K6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="L6" s="129"/>
-      <c r="M6" s="128" t="s">
+      <c r="L6" s="91"/>
+      <c r="M6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="N6" s="129"/>
-      <c r="O6" s="124"/>
-      <c r="P6" s="128" t="s">
+      <c r="N6" s="91"/>
+      <c r="O6" s="127"/>
+      <c r="P6" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="Q6" s="129"/>
-      <c r="R6" s="128" t="s">
+      <c r="Q6" s="91"/>
+      <c r="R6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="S6" s="129"/>
-      <c r="T6" s="128" t="s">
+      <c r="S6" s="91"/>
+      <c r="T6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="U6" s="129"/>
-      <c r="V6" s="112" t="s">
+      <c r="U6" s="91"/>
+      <c r="V6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="W6" s="127"/>
-      <c r="X6" s="113" t="s">
+      <c r="W6" s="94"/>
+      <c r="X6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="Y6" s="127"/>
-      <c r="Z6" s="113" t="s">
+      <c r="Y6" s="94"/>
+      <c r="Z6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AA6" s="114"/>
-      <c r="AB6" s="112" t="s">
+      <c r="AA6" s="93"/>
+      <c r="AB6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AC6" s="127"/>
-      <c r="AD6" s="113" t="s">
+      <c r="AC6" s="94"/>
+      <c r="AD6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AE6" s="127"/>
-      <c r="AF6" s="113" t="s">
+      <c r="AE6" s="94"/>
+      <c r="AF6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AG6" s="114"/>
-      <c r="AH6" s="112" t="s">
+      <c r="AG6" s="93"/>
+      <c r="AH6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AI6" s="127"/>
-      <c r="AJ6" s="113" t="s">
+      <c r="AI6" s="94"/>
+      <c r="AJ6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AK6" s="127"/>
-      <c r="AL6" s="113" t="s">
+      <c r="AK6" s="94"/>
+      <c r="AL6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AM6" s="114"/>
-      <c r="AN6" s="112" t="s">
+      <c r="AM6" s="93"/>
+      <c r="AN6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AO6" s="127"/>
-      <c r="AP6" s="113" t="s">
+      <c r="AO6" s="94"/>
+      <c r="AP6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AQ6" s="127"/>
-      <c r="AR6" s="113" t="s">
+      <c r="AQ6" s="94"/>
+      <c r="AR6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AS6" s="114"/>
-      <c r="AT6" s="112" t="s">
+      <c r="AS6" s="93"/>
+      <c r="AT6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AU6" s="127"/>
-      <c r="AV6" s="113" t="s">
+      <c r="AU6" s="94"/>
+      <c r="AV6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AW6" s="127"/>
-      <c r="AX6" s="113" t="s">
+      <c r="AW6" s="94"/>
+      <c r="AX6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AY6" s="114"/>
-      <c r="AZ6" s="112" t="s">
+      <c r="AY6" s="93"/>
+      <c r="AZ6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="BA6" s="127"/>
-      <c r="BB6" s="113" t="s">
+      <c r="BA6" s="94"/>
+      <c r="BB6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BC6" s="127"/>
-      <c r="BD6" s="113" t="s">
+      <c r="BC6" s="94"/>
+      <c r="BD6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BE6" s="114"/>
-      <c r="BF6" s="112" t="s">
+      <c r="BE6" s="93"/>
+      <c r="BF6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="BG6" s="127"/>
-      <c r="BH6" s="113" t="s">
+      <c r="BG6" s="94"/>
+      <c r="BH6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BI6" s="127"/>
-      <c r="BJ6" s="113" t="s">
+      <c r="BI6" s="94"/>
+      <c r="BJ6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BK6" s="114"/>
-      <c r="BL6" s="112" t="s">
+      <c r="BK6" s="93"/>
+      <c r="BL6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="BM6" s="127"/>
-      <c r="BN6" s="113" t="s">
+      <c r="BM6" s="94"/>
+      <c r="BN6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BO6" s="127"/>
-      <c r="BP6" s="113" t="s">
+      <c r="BO6" s="94"/>
+      <c r="BP6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BQ6" s="114"/>
+      <c r="BQ6" s="93"/>
     </row>
     <row r="7" spans="1:69" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
@@ -10552,38 +10552,6 @@
     </row>
   </sheetData>
   <mergeCells count="48">
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="X6:Y6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="R6:S6"/>
-    <mergeCell ref="AJ6:AK6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AD6:AE6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AT6:AU6"/>
-    <mergeCell ref="AR6:AS6"/>
-    <mergeCell ref="AP6:AQ6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="BD6:BE6"/>
-    <mergeCell ref="BB6:BC6"/>
-    <mergeCell ref="AZ6:BA6"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AV6:AW6"/>
-    <mergeCell ref="BN6:BO6"/>
-    <mergeCell ref="BL6:BM6"/>
-    <mergeCell ref="BJ6:BK6"/>
-    <mergeCell ref="BH6:BI6"/>
-    <mergeCell ref="BF6:BG6"/>
     <mergeCell ref="I4:N5"/>
     <mergeCell ref="V4:BQ4"/>
     <mergeCell ref="A4:A6"/>
@@ -10600,6 +10568,38 @@
     <mergeCell ref="C4:H5"/>
     <mergeCell ref="P4:U5"/>
     <mergeCell ref="O4:O6"/>
+    <mergeCell ref="BN6:BO6"/>
+    <mergeCell ref="BL6:BM6"/>
+    <mergeCell ref="BJ6:BK6"/>
+    <mergeCell ref="BH6:BI6"/>
+    <mergeCell ref="BF6:BG6"/>
+    <mergeCell ref="BD6:BE6"/>
+    <mergeCell ref="BB6:BC6"/>
+    <mergeCell ref="AZ6:BA6"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AV6:AW6"/>
+    <mergeCell ref="AT6:AU6"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="AP6:AQ6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="AJ6:AK6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AD6:AE6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="G6:H6"/>
   </mergeCells>
   <conditionalFormatting sqref="D1:D1048576 F1:F1048576 H1:H1048576 J1:J1048576 L1:L1048576 N1:N1048576 Q1:Q1048576 S1:S1048576 U1:U1048576 W1:W1048576 Y1:Y1048576 AA1:AA1048576 AC1:AC1048576 AE1:AE1048576 AG1:AG1048576 AI1:AI1048576 AK1:AK1048576 AM1:AM1048576 AO1:AO1048576 AQ1:AQ1048576 AS1:AS1048576 AU1:AU1048576 AW1:AW1048576 AY1:AY1048576 BA1:BA1048576 BC1:BC1048576 BE1:BE1048576 BG1:BG1048576 BI1:BI1048576 BK1:BK1048576 BM1:BM1048576 BO1:BO1048576 BQ1:BQ1048576">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">

</xml_diff>

<commit_message>
tmp: Save updated PEB test workbooks and run history
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
+++ b/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\tests\PersonalEventBuilder\Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAE89B2B-98C1-463D-8A36-62BA6DB564C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A29B197C-AF66-4156-9CAF-C70CE7114D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2268,125 +2268,125 @@
     <xf numFmtId="164" fontId="38" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="161">
@@ -4075,7 +4075,7 @@
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B9">
-    <cfRule type="duplicateValues" dxfId="2" priority="20782"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="20783"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -4177,311 +4177,311 @@
     </row>
     <row r="3" spans="1:69" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="109" t="s">
+      <c r="A4" s="103" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="117"/>
-      <c r="C4" s="109" t="s">
+      <c r="B4" s="111"/>
+      <c r="C4" s="103" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="118"/>
-      <c r="E4" s="118"/>
-      <c r="F4" s="118"/>
-      <c r="G4" s="118"/>
-      <c r="H4" s="119"/>
-      <c r="I4" s="96" t="s">
+      <c r="D4" s="115"/>
+      <c r="E4" s="115"/>
+      <c r="F4" s="115"/>
+      <c r="G4" s="115"/>
+      <c r="H4" s="116"/>
+      <c r="I4" s="90" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="97"/>
-      <c r="K4" s="98"/>
-      <c r="L4" s="99"/>
-      <c r="M4" s="99"/>
-      <c r="N4" s="100"/>
-      <c r="O4" s="124" t="s">
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
+      <c r="L4" s="93"/>
+      <c r="M4" s="93"/>
+      <c r="N4" s="94"/>
+      <c r="O4" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="P4" s="123" t="s">
+      <c r="P4" s="120" t="s">
         <v>24</v>
       </c>
-      <c r="Q4" s="124"/>
-      <c r="R4" s="124"/>
-      <c r="S4" s="124"/>
-      <c r="T4" s="124"/>
-      <c r="U4" s="125"/>
-      <c r="V4" s="106" t="s">
+      <c r="Q4" s="121"/>
+      <c r="R4" s="121"/>
+      <c r="S4" s="121"/>
+      <c r="T4" s="121"/>
+      <c r="U4" s="122"/>
+      <c r="V4" s="100" t="s">
         <v>25</v>
       </c>
-      <c r="W4" s="107"/>
-      <c r="X4" s="107"/>
-      <c r="Y4" s="107"/>
-      <c r="Z4" s="107"/>
-      <c r="AA4" s="107"/>
-      <c r="AB4" s="107"/>
-      <c r="AC4" s="107"/>
-      <c r="AD4" s="107"/>
-      <c r="AE4" s="107"/>
-      <c r="AF4" s="107"/>
-      <c r="AG4" s="107"/>
-      <c r="AH4" s="107"/>
-      <c r="AI4" s="107"/>
-      <c r="AJ4" s="107"/>
-      <c r="AK4" s="107"/>
-      <c r="AL4" s="107"/>
-      <c r="AM4" s="107"/>
-      <c r="AN4" s="107"/>
-      <c r="AO4" s="107"/>
-      <c r="AP4" s="107"/>
-      <c r="AQ4" s="107"/>
-      <c r="AR4" s="107"/>
-      <c r="AS4" s="107"/>
-      <c r="AT4" s="107"/>
-      <c r="AU4" s="107"/>
-      <c r="AV4" s="107"/>
-      <c r="AW4" s="107"/>
-      <c r="AX4" s="107"/>
-      <c r="AY4" s="107"/>
-      <c r="AZ4" s="107"/>
-      <c r="BA4" s="107"/>
-      <c r="BB4" s="107"/>
-      <c r="BC4" s="107"/>
-      <c r="BD4" s="107"/>
-      <c r="BE4" s="107"/>
-      <c r="BF4" s="107"/>
-      <c r="BG4" s="107"/>
-      <c r="BH4" s="107"/>
-      <c r="BI4" s="107"/>
-      <c r="BJ4" s="107"/>
-      <c r="BK4" s="107"/>
-      <c r="BL4" s="107"/>
-      <c r="BM4" s="107"/>
-      <c r="BN4" s="107"/>
-      <c r="BO4" s="107"/>
-      <c r="BP4" s="107"/>
-      <c r="BQ4" s="108"/>
+      <c r="W4" s="101"/>
+      <c r="X4" s="101"/>
+      <c r="Y4" s="101"/>
+      <c r="Z4" s="101"/>
+      <c r="AA4" s="101"/>
+      <c r="AB4" s="101"/>
+      <c r="AC4" s="101"/>
+      <c r="AD4" s="101"/>
+      <c r="AE4" s="101"/>
+      <c r="AF4" s="101"/>
+      <c r="AG4" s="101"/>
+      <c r="AH4" s="101"/>
+      <c r="AI4" s="101"/>
+      <c r="AJ4" s="101"/>
+      <c r="AK4" s="101"/>
+      <c r="AL4" s="101"/>
+      <c r="AM4" s="101"/>
+      <c r="AN4" s="101"/>
+      <c r="AO4" s="101"/>
+      <c r="AP4" s="101"/>
+      <c r="AQ4" s="101"/>
+      <c r="AR4" s="101"/>
+      <c r="AS4" s="101"/>
+      <c r="AT4" s="101"/>
+      <c r="AU4" s="101"/>
+      <c r="AV4" s="101"/>
+      <c r="AW4" s="101"/>
+      <c r="AX4" s="101"/>
+      <c r="AY4" s="101"/>
+      <c r="AZ4" s="101"/>
+      <c r="BA4" s="101"/>
+      <c r="BB4" s="101"/>
+      <c r="BC4" s="101"/>
+      <c r="BD4" s="101"/>
+      <c r="BE4" s="101"/>
+      <c r="BF4" s="101"/>
+      <c r="BG4" s="101"/>
+      <c r="BH4" s="101"/>
+      <c r="BI4" s="101"/>
+      <c r="BJ4" s="101"/>
+      <c r="BK4" s="101"/>
+      <c r="BL4" s="101"/>
+      <c r="BM4" s="101"/>
+      <c r="BN4" s="101"/>
+      <c r="BO4" s="101"/>
+      <c r="BP4" s="101"/>
+      <c r="BQ4" s="102"/>
     </row>
     <row r="5" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="110"/>
-      <c r="B5" s="117"/>
-      <c r="C5" s="120"/>
-      <c r="D5" s="121"/>
-      <c r="E5" s="121"/>
-      <c r="F5" s="121"/>
-      <c r="G5" s="121"/>
-      <c r="H5" s="122"/>
-      <c r="I5" s="101"/>
-      <c r="J5" s="102"/>
-      <c r="K5" s="103"/>
-      <c r="L5" s="104"/>
-      <c r="M5" s="104"/>
-      <c r="N5" s="105"/>
-      <c r="O5" s="129"/>
-      <c r="P5" s="126"/>
-      <c r="Q5" s="127"/>
-      <c r="R5" s="127"/>
-      <c r="S5" s="127"/>
-      <c r="T5" s="127"/>
-      <c r="U5" s="128"/>
-      <c r="V5" s="111" t="s">
+      <c r="A5" s="104"/>
+      <c r="B5" s="111"/>
+      <c r="C5" s="117"/>
+      <c r="D5" s="118"/>
+      <c r="E5" s="118"/>
+      <c r="F5" s="118"/>
+      <c r="G5" s="118"/>
+      <c r="H5" s="119"/>
+      <c r="I5" s="95"/>
+      <c r="J5" s="96"/>
+      <c r="K5" s="97"/>
+      <c r="L5" s="98"/>
+      <c r="M5" s="98"/>
+      <c r="N5" s="99"/>
+      <c r="O5" s="126"/>
+      <c r="P5" s="123"/>
+      <c r="Q5" s="124"/>
+      <c r="R5" s="124"/>
+      <c r="S5" s="124"/>
+      <c r="T5" s="124"/>
+      <c r="U5" s="125"/>
+      <c r="V5" s="105" t="s">
         <v>19</v>
       </c>
-      <c r="W5" s="112"/>
-      <c r="X5" s="112"/>
-      <c r="Y5" s="112"/>
-      <c r="Z5" s="112"/>
-      <c r="AA5" s="113"/>
-      <c r="AB5" s="114" t="s">
+      <c r="W5" s="106"/>
+      <c r="X5" s="106"/>
+      <c r="Y5" s="106"/>
+      <c r="Z5" s="106"/>
+      <c r="AA5" s="107"/>
+      <c r="AB5" s="108" t="s">
         <v>18</v>
       </c>
-      <c r="AC5" s="115"/>
-      <c r="AD5" s="115"/>
-      <c r="AE5" s="115"/>
-      <c r="AF5" s="115"/>
-      <c r="AG5" s="116"/>
-      <c r="AH5" s="114" t="s">
+      <c r="AC5" s="109"/>
+      <c r="AD5" s="109"/>
+      <c r="AE5" s="109"/>
+      <c r="AF5" s="109"/>
+      <c r="AG5" s="110"/>
+      <c r="AH5" s="108" t="s">
         <v>26</v>
       </c>
-      <c r="AI5" s="115"/>
-      <c r="AJ5" s="115"/>
-      <c r="AK5" s="115"/>
-      <c r="AL5" s="115"/>
-      <c r="AM5" s="116"/>
-      <c r="AN5" s="114" t="s">
+      <c r="AI5" s="109"/>
+      <c r="AJ5" s="109"/>
+      <c r="AK5" s="109"/>
+      <c r="AL5" s="109"/>
+      <c r="AM5" s="110"/>
+      <c r="AN5" s="108" t="s">
         <v>27</v>
       </c>
-      <c r="AO5" s="115"/>
-      <c r="AP5" s="115"/>
-      <c r="AQ5" s="115"/>
-      <c r="AR5" s="115"/>
-      <c r="AS5" s="116"/>
-      <c r="AT5" s="114" t="s">
+      <c r="AO5" s="109"/>
+      <c r="AP5" s="109"/>
+      <c r="AQ5" s="109"/>
+      <c r="AR5" s="109"/>
+      <c r="AS5" s="110"/>
+      <c r="AT5" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="AU5" s="115"/>
-      <c r="AV5" s="115"/>
-      <c r="AW5" s="115"/>
-      <c r="AX5" s="115"/>
-      <c r="AY5" s="116"/>
-      <c r="AZ5" s="114" t="s">
+      <c r="AU5" s="109"/>
+      <c r="AV5" s="109"/>
+      <c r="AW5" s="109"/>
+      <c r="AX5" s="109"/>
+      <c r="AY5" s="110"/>
+      <c r="AZ5" s="108" t="s">
         <v>29</v>
       </c>
-      <c r="BA5" s="115"/>
-      <c r="BB5" s="115"/>
-      <c r="BC5" s="115"/>
-      <c r="BD5" s="115"/>
-      <c r="BE5" s="116"/>
-      <c r="BF5" s="114" t="s">
+      <c r="BA5" s="109"/>
+      <c r="BB5" s="109"/>
+      <c r="BC5" s="109"/>
+      <c r="BD5" s="109"/>
+      <c r="BE5" s="110"/>
+      <c r="BF5" s="108" t="s">
         <v>30</v>
       </c>
-      <c r="BG5" s="115"/>
-      <c r="BH5" s="115"/>
-      <c r="BI5" s="115"/>
-      <c r="BJ5" s="115"/>
-      <c r="BK5" s="116"/>
-      <c r="BL5" s="96" t="s">
+      <c r="BG5" s="109"/>
+      <c r="BH5" s="109"/>
+      <c r="BI5" s="109"/>
+      <c r="BJ5" s="109"/>
+      <c r="BK5" s="110"/>
+      <c r="BL5" s="90" t="s">
         <v>31</v>
       </c>
-      <c r="BM5" s="98"/>
-      <c r="BN5" s="98"/>
-      <c r="BO5" s="99"/>
-      <c r="BP5" s="99"/>
-      <c r="BQ5" s="100"/>
+      <c r="BM5" s="92"/>
+      <c r="BN5" s="92"/>
+      <c r="BO5" s="93"/>
+      <c r="BP5" s="93"/>
+      <c r="BQ5" s="94"/>
     </row>
     <row r="6" spans="1:69" ht="103.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="110"/>
-      <c r="B6" s="95"/>
-      <c r="C6" s="90" t="s">
+      <c r="A6" s="104"/>
+      <c r="B6" s="112"/>
+      <c r="C6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="91"/>
-      <c r="E6" s="90" t="s">
+      <c r="D6" s="129"/>
+      <c r="E6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="91"/>
-      <c r="G6" s="90" t="s">
+      <c r="F6" s="129"/>
+      <c r="G6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="91"/>
-      <c r="I6" s="90" t="s">
+      <c r="H6" s="129"/>
+      <c r="I6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="J6" s="91"/>
-      <c r="K6" s="90" t="s">
+      <c r="J6" s="129"/>
+      <c r="K6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="L6" s="91"/>
-      <c r="M6" s="90" t="s">
+      <c r="L6" s="129"/>
+      <c r="M6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="N6" s="91"/>
-      <c r="O6" s="127"/>
-      <c r="P6" s="90" t="s">
+      <c r="N6" s="129"/>
+      <c r="O6" s="124"/>
+      <c r="P6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="Q6" s="91"/>
-      <c r="R6" s="90" t="s">
+      <c r="Q6" s="129"/>
+      <c r="R6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="S6" s="91"/>
-      <c r="T6" s="90" t="s">
+      <c r="S6" s="129"/>
+      <c r="T6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="U6" s="91"/>
-      <c r="V6" s="95" t="s">
+      <c r="U6" s="129"/>
+      <c r="V6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="W6" s="94"/>
-      <c r="X6" s="92" t="s">
+      <c r="W6" s="127"/>
+      <c r="X6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="Y6" s="94"/>
-      <c r="Z6" s="92" t="s">
+      <c r="Y6" s="127"/>
+      <c r="Z6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AA6" s="93"/>
-      <c r="AB6" s="95" t="s">
+      <c r="AA6" s="114"/>
+      <c r="AB6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AC6" s="94"/>
-      <c r="AD6" s="92" t="s">
+      <c r="AC6" s="127"/>
+      <c r="AD6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AE6" s="94"/>
-      <c r="AF6" s="92" t="s">
+      <c r="AE6" s="127"/>
+      <c r="AF6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AG6" s="93"/>
-      <c r="AH6" s="95" t="s">
+      <c r="AG6" s="114"/>
+      <c r="AH6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AI6" s="94"/>
-      <c r="AJ6" s="92" t="s">
+      <c r="AI6" s="127"/>
+      <c r="AJ6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AK6" s="94"/>
-      <c r="AL6" s="92" t="s">
+      <c r="AK6" s="127"/>
+      <c r="AL6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AM6" s="93"/>
-      <c r="AN6" s="95" t="s">
+      <c r="AM6" s="114"/>
+      <c r="AN6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AO6" s="94"/>
-      <c r="AP6" s="92" t="s">
+      <c r="AO6" s="127"/>
+      <c r="AP6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AQ6" s="94"/>
-      <c r="AR6" s="92" t="s">
+      <c r="AQ6" s="127"/>
+      <c r="AR6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AS6" s="93"/>
-      <c r="AT6" s="95" t="s">
+      <c r="AS6" s="114"/>
+      <c r="AT6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AU6" s="94"/>
-      <c r="AV6" s="92" t="s">
+      <c r="AU6" s="127"/>
+      <c r="AV6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AW6" s="94"/>
-      <c r="AX6" s="92" t="s">
+      <c r="AW6" s="127"/>
+      <c r="AX6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AY6" s="93"/>
-      <c r="AZ6" s="95" t="s">
+      <c r="AY6" s="114"/>
+      <c r="AZ6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BA6" s="94"/>
-      <c r="BB6" s="92" t="s">
+      <c r="BA6" s="127"/>
+      <c r="BB6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BC6" s="94"/>
-      <c r="BD6" s="92" t="s">
+      <c r="BC6" s="127"/>
+      <c r="BD6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BE6" s="93"/>
-      <c r="BF6" s="95" t="s">
+      <c r="BE6" s="114"/>
+      <c r="BF6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BG6" s="94"/>
-      <c r="BH6" s="92" t="s">
+      <c r="BG6" s="127"/>
+      <c r="BH6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BI6" s="94"/>
-      <c r="BJ6" s="92" t="s">
+      <c r="BI6" s="127"/>
+      <c r="BJ6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BK6" s="93"/>
-      <c r="BL6" s="95" t="s">
+      <c r="BK6" s="114"/>
+      <c r="BL6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BM6" s="94"/>
-      <c r="BN6" s="92" t="s">
+      <c r="BM6" s="127"/>
+      <c r="BN6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BO6" s="94"/>
-      <c r="BP6" s="92" t="s">
+      <c r="BO6" s="127"/>
+      <c r="BP6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BQ6" s="93"/>
+      <c r="BQ6" s="114"/>
     </row>
     <row r="7" spans="1:69" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
@@ -10552,6 +10552,38 @@
     </row>
   </sheetData>
   <mergeCells count="48">
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="AJ6:AK6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AD6:AE6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AT6:AU6"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="AP6:AQ6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="BD6:BE6"/>
+    <mergeCell ref="BB6:BC6"/>
+    <mergeCell ref="AZ6:BA6"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AV6:AW6"/>
+    <mergeCell ref="BN6:BO6"/>
+    <mergeCell ref="BL6:BM6"/>
+    <mergeCell ref="BJ6:BK6"/>
+    <mergeCell ref="BH6:BI6"/>
+    <mergeCell ref="BF6:BG6"/>
     <mergeCell ref="I4:N5"/>
     <mergeCell ref="V4:BQ4"/>
     <mergeCell ref="A4:A6"/>
@@ -10568,38 +10600,6 @@
     <mergeCell ref="C4:H5"/>
     <mergeCell ref="P4:U5"/>
     <mergeCell ref="O4:O6"/>
-    <mergeCell ref="BN6:BO6"/>
-    <mergeCell ref="BL6:BM6"/>
-    <mergeCell ref="BJ6:BK6"/>
-    <mergeCell ref="BH6:BI6"/>
-    <mergeCell ref="BF6:BG6"/>
-    <mergeCell ref="BD6:BE6"/>
-    <mergeCell ref="BB6:BC6"/>
-    <mergeCell ref="AZ6:BA6"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AV6:AW6"/>
-    <mergeCell ref="AT6:AU6"/>
-    <mergeCell ref="AR6:AS6"/>
-    <mergeCell ref="AP6:AQ6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="AJ6:AK6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AD6:AE6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="X6:Y6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="R6:S6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="G6:H6"/>
   </mergeCells>
   <conditionalFormatting sqref="D1:D1048576 F1:F1048576 H1:H1048576 J1:J1048576 L1:L1048576 N1:N1048576 Q1:Q1048576 S1:S1048576 U1:U1048576 W1:W1048576 Y1:Y1048576 AA1:AA1048576 AC1:AC1048576 AE1:AE1048576 AG1:AG1048576 AI1:AI1048576 AK1:AK1048576 AM1:AM1048576 AO1:AO1048576 AQ1:AQ1048576 AS1:AS1048576 AU1:AU1048576 AW1:AW1048576 AY1:AY1048576 BA1:BA1048576 BC1:BC1048576 BE1:BE1048576 BG1:BG1048576 BI1:BI1048576 BK1:BK1048576 BM1:BM1048576 BO1:BO1048576 BQ1:BQ1048576">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">

</xml_diff>

<commit_message>
Unify Movement target and add calculated scenario expectations
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
+++ b/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\tests\PersonalEventBuilder\Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A29B197C-AF66-4156-9CAF-C70CE7114D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33261F51-14A9-4980-938D-C463F45BDFB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2268,6 +2268,24 @@
     <xf numFmtId="164" fontId="38" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2334,15 +2352,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2378,15 +2387,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="161">
@@ -4075,7 +4075,7 @@
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B9">
-    <cfRule type="duplicateValues" dxfId="2" priority="20783"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="20784"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -4177,311 +4177,311 @@
     </row>
     <row r="3" spans="1:69" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="103" t="s">
+      <c r="A4" s="109" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="111"/>
-      <c r="C4" s="103" t="s">
+      <c r="B4" s="117"/>
+      <c r="C4" s="109" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="115"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="116"/>
-      <c r="I4" s="90" t="s">
+      <c r="D4" s="118"/>
+      <c r="E4" s="118"/>
+      <c r="F4" s="118"/>
+      <c r="G4" s="118"/>
+      <c r="H4" s="119"/>
+      <c r="I4" s="96" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
-      <c r="L4" s="93"/>
-      <c r="M4" s="93"/>
-      <c r="N4" s="94"/>
-      <c r="O4" s="121" t="s">
+      <c r="J4" s="97"/>
+      <c r="K4" s="98"/>
+      <c r="L4" s="99"/>
+      <c r="M4" s="99"/>
+      <c r="N4" s="100"/>
+      <c r="O4" s="124" t="s">
         <v>23</v>
       </c>
-      <c r="P4" s="120" t="s">
+      <c r="P4" s="123" t="s">
         <v>24</v>
       </c>
-      <c r="Q4" s="121"/>
-      <c r="R4" s="121"/>
-      <c r="S4" s="121"/>
-      <c r="T4" s="121"/>
-      <c r="U4" s="122"/>
-      <c r="V4" s="100" t="s">
+      <c r="Q4" s="124"/>
+      <c r="R4" s="124"/>
+      <c r="S4" s="124"/>
+      <c r="T4" s="124"/>
+      <c r="U4" s="125"/>
+      <c r="V4" s="106" t="s">
         <v>25</v>
       </c>
-      <c r="W4" s="101"/>
-      <c r="X4" s="101"/>
-      <c r="Y4" s="101"/>
-      <c r="Z4" s="101"/>
-      <c r="AA4" s="101"/>
-      <c r="AB4" s="101"/>
-      <c r="AC4" s="101"/>
-      <c r="AD4" s="101"/>
-      <c r="AE4" s="101"/>
-      <c r="AF4" s="101"/>
-      <c r="AG4" s="101"/>
-      <c r="AH4" s="101"/>
-      <c r="AI4" s="101"/>
-      <c r="AJ4" s="101"/>
-      <c r="AK4" s="101"/>
-      <c r="AL4" s="101"/>
-      <c r="AM4" s="101"/>
-      <c r="AN4" s="101"/>
-      <c r="AO4" s="101"/>
-      <c r="AP4" s="101"/>
-      <c r="AQ4" s="101"/>
-      <c r="AR4" s="101"/>
-      <c r="AS4" s="101"/>
-      <c r="AT4" s="101"/>
-      <c r="AU4" s="101"/>
-      <c r="AV4" s="101"/>
-      <c r="AW4" s="101"/>
-      <c r="AX4" s="101"/>
-      <c r="AY4" s="101"/>
-      <c r="AZ4" s="101"/>
-      <c r="BA4" s="101"/>
-      <c r="BB4" s="101"/>
-      <c r="BC4" s="101"/>
-      <c r="BD4" s="101"/>
-      <c r="BE4" s="101"/>
-      <c r="BF4" s="101"/>
-      <c r="BG4" s="101"/>
-      <c r="BH4" s="101"/>
-      <c r="BI4" s="101"/>
-      <c r="BJ4" s="101"/>
-      <c r="BK4" s="101"/>
-      <c r="BL4" s="101"/>
-      <c r="BM4" s="101"/>
-      <c r="BN4" s="101"/>
-      <c r="BO4" s="101"/>
-      <c r="BP4" s="101"/>
-      <c r="BQ4" s="102"/>
+      <c r="W4" s="107"/>
+      <c r="X4" s="107"/>
+      <c r="Y4" s="107"/>
+      <c r="Z4" s="107"/>
+      <c r="AA4" s="107"/>
+      <c r="AB4" s="107"/>
+      <c r="AC4" s="107"/>
+      <c r="AD4" s="107"/>
+      <c r="AE4" s="107"/>
+      <c r="AF4" s="107"/>
+      <c r="AG4" s="107"/>
+      <c r="AH4" s="107"/>
+      <c r="AI4" s="107"/>
+      <c r="AJ4" s="107"/>
+      <c r="AK4" s="107"/>
+      <c r="AL4" s="107"/>
+      <c r="AM4" s="107"/>
+      <c r="AN4" s="107"/>
+      <c r="AO4" s="107"/>
+      <c r="AP4" s="107"/>
+      <c r="AQ4" s="107"/>
+      <c r="AR4" s="107"/>
+      <c r="AS4" s="107"/>
+      <c r="AT4" s="107"/>
+      <c r="AU4" s="107"/>
+      <c r="AV4" s="107"/>
+      <c r="AW4" s="107"/>
+      <c r="AX4" s="107"/>
+      <c r="AY4" s="107"/>
+      <c r="AZ4" s="107"/>
+      <c r="BA4" s="107"/>
+      <c r="BB4" s="107"/>
+      <c r="BC4" s="107"/>
+      <c r="BD4" s="107"/>
+      <c r="BE4" s="107"/>
+      <c r="BF4" s="107"/>
+      <c r="BG4" s="107"/>
+      <c r="BH4" s="107"/>
+      <c r="BI4" s="107"/>
+      <c r="BJ4" s="107"/>
+      <c r="BK4" s="107"/>
+      <c r="BL4" s="107"/>
+      <c r="BM4" s="107"/>
+      <c r="BN4" s="107"/>
+      <c r="BO4" s="107"/>
+      <c r="BP4" s="107"/>
+      <c r="BQ4" s="108"/>
     </row>
     <row r="5" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="104"/>
-      <c r="B5" s="111"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="118"/>
-      <c r="E5" s="118"/>
-      <c r="F5" s="118"/>
-      <c r="G5" s="118"/>
-      <c r="H5" s="119"/>
-      <c r="I5" s="95"/>
-      <c r="J5" s="96"/>
-      <c r="K5" s="97"/>
-      <c r="L5" s="98"/>
-      <c r="M5" s="98"/>
-      <c r="N5" s="99"/>
-      <c r="O5" s="126"/>
-      <c r="P5" s="123"/>
-      <c r="Q5" s="124"/>
-      <c r="R5" s="124"/>
-      <c r="S5" s="124"/>
-      <c r="T5" s="124"/>
-      <c r="U5" s="125"/>
-      <c r="V5" s="105" t="s">
+      <c r="A5" s="110"/>
+      <c r="B5" s="117"/>
+      <c r="C5" s="120"/>
+      <c r="D5" s="121"/>
+      <c r="E5" s="121"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="121"/>
+      <c r="H5" s="122"/>
+      <c r="I5" s="101"/>
+      <c r="J5" s="102"/>
+      <c r="K5" s="103"/>
+      <c r="L5" s="104"/>
+      <c r="M5" s="104"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="129"/>
+      <c r="P5" s="126"/>
+      <c r="Q5" s="127"/>
+      <c r="R5" s="127"/>
+      <c r="S5" s="127"/>
+      <c r="T5" s="127"/>
+      <c r="U5" s="128"/>
+      <c r="V5" s="111" t="s">
         <v>19</v>
       </c>
-      <c r="W5" s="106"/>
-      <c r="X5" s="106"/>
-      <c r="Y5" s="106"/>
-      <c r="Z5" s="106"/>
-      <c r="AA5" s="107"/>
-      <c r="AB5" s="108" t="s">
+      <c r="W5" s="112"/>
+      <c r="X5" s="112"/>
+      <c r="Y5" s="112"/>
+      <c r="Z5" s="112"/>
+      <c r="AA5" s="113"/>
+      <c r="AB5" s="114" t="s">
         <v>18</v>
       </c>
-      <c r="AC5" s="109"/>
-      <c r="AD5" s="109"/>
-      <c r="AE5" s="109"/>
-      <c r="AF5" s="109"/>
-      <c r="AG5" s="110"/>
-      <c r="AH5" s="108" t="s">
+      <c r="AC5" s="115"/>
+      <c r="AD5" s="115"/>
+      <c r="AE5" s="115"/>
+      <c r="AF5" s="115"/>
+      <c r="AG5" s="116"/>
+      <c r="AH5" s="114" t="s">
         <v>26</v>
       </c>
-      <c r="AI5" s="109"/>
-      <c r="AJ5" s="109"/>
-      <c r="AK5" s="109"/>
-      <c r="AL5" s="109"/>
-      <c r="AM5" s="110"/>
-      <c r="AN5" s="108" t="s">
+      <c r="AI5" s="115"/>
+      <c r="AJ5" s="115"/>
+      <c r="AK5" s="115"/>
+      <c r="AL5" s="115"/>
+      <c r="AM5" s="116"/>
+      <c r="AN5" s="114" t="s">
         <v>27</v>
       </c>
-      <c r="AO5" s="109"/>
-      <c r="AP5" s="109"/>
-      <c r="AQ5" s="109"/>
-      <c r="AR5" s="109"/>
-      <c r="AS5" s="110"/>
-      <c r="AT5" s="108" t="s">
+      <c r="AO5" s="115"/>
+      <c r="AP5" s="115"/>
+      <c r="AQ5" s="115"/>
+      <c r="AR5" s="115"/>
+      <c r="AS5" s="116"/>
+      <c r="AT5" s="114" t="s">
         <v>28</v>
       </c>
-      <c r="AU5" s="109"/>
-      <c r="AV5" s="109"/>
-      <c r="AW5" s="109"/>
-      <c r="AX5" s="109"/>
-      <c r="AY5" s="110"/>
-      <c r="AZ5" s="108" t="s">
+      <c r="AU5" s="115"/>
+      <c r="AV5" s="115"/>
+      <c r="AW5" s="115"/>
+      <c r="AX5" s="115"/>
+      <c r="AY5" s="116"/>
+      <c r="AZ5" s="114" t="s">
         <v>29</v>
       </c>
-      <c r="BA5" s="109"/>
-      <c r="BB5" s="109"/>
-      <c r="BC5" s="109"/>
-      <c r="BD5" s="109"/>
-      <c r="BE5" s="110"/>
-      <c r="BF5" s="108" t="s">
+      <c r="BA5" s="115"/>
+      <c r="BB5" s="115"/>
+      <c r="BC5" s="115"/>
+      <c r="BD5" s="115"/>
+      <c r="BE5" s="116"/>
+      <c r="BF5" s="114" t="s">
         <v>30</v>
       </c>
-      <c r="BG5" s="109"/>
-      <c r="BH5" s="109"/>
-      <c r="BI5" s="109"/>
-      <c r="BJ5" s="109"/>
-      <c r="BK5" s="110"/>
-      <c r="BL5" s="90" t="s">
+      <c r="BG5" s="115"/>
+      <c r="BH5" s="115"/>
+      <c r="BI5" s="115"/>
+      <c r="BJ5" s="115"/>
+      <c r="BK5" s="116"/>
+      <c r="BL5" s="96" t="s">
         <v>31</v>
       </c>
-      <c r="BM5" s="92"/>
-      <c r="BN5" s="92"/>
-      <c r="BO5" s="93"/>
-      <c r="BP5" s="93"/>
-      <c r="BQ5" s="94"/>
+      <c r="BM5" s="98"/>
+      <c r="BN5" s="98"/>
+      <c r="BO5" s="99"/>
+      <c r="BP5" s="99"/>
+      <c r="BQ5" s="100"/>
     </row>
     <row r="6" spans="1:69" ht="103.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="104"/>
-      <c r="B6" s="112"/>
-      <c r="C6" s="128" t="s">
+      <c r="A6" s="110"/>
+      <c r="B6" s="95"/>
+      <c r="C6" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="129"/>
-      <c r="E6" s="128" t="s">
+      <c r="D6" s="91"/>
+      <c r="E6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="129"/>
-      <c r="G6" s="128" t="s">
+      <c r="F6" s="91"/>
+      <c r="G6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="129"/>
-      <c r="I6" s="128" t="s">
+      <c r="H6" s="91"/>
+      <c r="I6" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="J6" s="129"/>
-      <c r="K6" s="128" t="s">
+      <c r="J6" s="91"/>
+      <c r="K6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="L6" s="129"/>
-      <c r="M6" s="128" t="s">
+      <c r="L6" s="91"/>
+      <c r="M6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="N6" s="129"/>
-      <c r="O6" s="124"/>
-      <c r="P6" s="128" t="s">
+      <c r="N6" s="91"/>
+      <c r="O6" s="127"/>
+      <c r="P6" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="Q6" s="129"/>
-      <c r="R6" s="128" t="s">
+      <c r="Q6" s="91"/>
+      <c r="R6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="S6" s="129"/>
-      <c r="T6" s="128" t="s">
+      <c r="S6" s="91"/>
+      <c r="T6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="U6" s="129"/>
-      <c r="V6" s="112" t="s">
+      <c r="U6" s="91"/>
+      <c r="V6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="W6" s="127"/>
-      <c r="X6" s="113" t="s">
+      <c r="W6" s="94"/>
+      <c r="X6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="Y6" s="127"/>
-      <c r="Z6" s="113" t="s">
+      <c r="Y6" s="94"/>
+      <c r="Z6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AA6" s="114"/>
-      <c r="AB6" s="112" t="s">
+      <c r="AA6" s="93"/>
+      <c r="AB6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AC6" s="127"/>
-      <c r="AD6" s="113" t="s">
+      <c r="AC6" s="94"/>
+      <c r="AD6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AE6" s="127"/>
-      <c r="AF6" s="113" t="s">
+      <c r="AE6" s="94"/>
+      <c r="AF6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AG6" s="114"/>
-      <c r="AH6" s="112" t="s">
+      <c r="AG6" s="93"/>
+      <c r="AH6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AI6" s="127"/>
-      <c r="AJ6" s="113" t="s">
+      <c r="AI6" s="94"/>
+      <c r="AJ6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AK6" s="127"/>
-      <c r="AL6" s="113" t="s">
+      <c r="AK6" s="94"/>
+      <c r="AL6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AM6" s="114"/>
-      <c r="AN6" s="112" t="s">
+      <c r="AM6" s="93"/>
+      <c r="AN6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AO6" s="127"/>
-      <c r="AP6" s="113" t="s">
+      <c r="AO6" s="94"/>
+      <c r="AP6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AQ6" s="127"/>
-      <c r="AR6" s="113" t="s">
+      <c r="AQ6" s="94"/>
+      <c r="AR6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AS6" s="114"/>
-      <c r="AT6" s="112" t="s">
+      <c r="AS6" s="93"/>
+      <c r="AT6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AU6" s="127"/>
-      <c r="AV6" s="113" t="s">
+      <c r="AU6" s="94"/>
+      <c r="AV6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AW6" s="127"/>
-      <c r="AX6" s="113" t="s">
+      <c r="AW6" s="94"/>
+      <c r="AX6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AY6" s="114"/>
-      <c r="AZ6" s="112" t="s">
+      <c r="AY6" s="93"/>
+      <c r="AZ6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="BA6" s="127"/>
-      <c r="BB6" s="113" t="s">
+      <c r="BA6" s="94"/>
+      <c r="BB6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BC6" s="127"/>
-      <c r="BD6" s="113" t="s">
+      <c r="BC6" s="94"/>
+      <c r="BD6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BE6" s="114"/>
-      <c r="BF6" s="112" t="s">
+      <c r="BE6" s="93"/>
+      <c r="BF6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="BG6" s="127"/>
-      <c r="BH6" s="113" t="s">
+      <c r="BG6" s="94"/>
+      <c r="BH6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BI6" s="127"/>
-      <c r="BJ6" s="113" t="s">
+      <c r="BI6" s="94"/>
+      <c r="BJ6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BK6" s="114"/>
-      <c r="BL6" s="112" t="s">
+      <c r="BK6" s="93"/>
+      <c r="BL6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="BM6" s="127"/>
-      <c r="BN6" s="113" t="s">
+      <c r="BM6" s="94"/>
+      <c r="BN6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BO6" s="127"/>
-      <c r="BP6" s="113" t="s">
+      <c r="BO6" s="94"/>
+      <c r="BP6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BQ6" s="114"/>
+      <c r="BQ6" s="93"/>
     </row>
     <row r="7" spans="1:69" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
@@ -10552,38 +10552,6 @@
     </row>
   </sheetData>
   <mergeCells count="48">
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="X6:Y6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="R6:S6"/>
-    <mergeCell ref="AJ6:AK6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AD6:AE6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AT6:AU6"/>
-    <mergeCell ref="AR6:AS6"/>
-    <mergeCell ref="AP6:AQ6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="BD6:BE6"/>
-    <mergeCell ref="BB6:BC6"/>
-    <mergeCell ref="AZ6:BA6"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AV6:AW6"/>
-    <mergeCell ref="BN6:BO6"/>
-    <mergeCell ref="BL6:BM6"/>
-    <mergeCell ref="BJ6:BK6"/>
-    <mergeCell ref="BH6:BI6"/>
-    <mergeCell ref="BF6:BG6"/>
     <mergeCell ref="I4:N5"/>
     <mergeCell ref="V4:BQ4"/>
     <mergeCell ref="A4:A6"/>
@@ -10600,6 +10568,38 @@
     <mergeCell ref="C4:H5"/>
     <mergeCell ref="P4:U5"/>
     <mergeCell ref="O4:O6"/>
+    <mergeCell ref="BN6:BO6"/>
+    <mergeCell ref="BL6:BM6"/>
+    <mergeCell ref="BJ6:BK6"/>
+    <mergeCell ref="BH6:BI6"/>
+    <mergeCell ref="BF6:BG6"/>
+    <mergeCell ref="BD6:BE6"/>
+    <mergeCell ref="BB6:BC6"/>
+    <mergeCell ref="AZ6:BA6"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AV6:AW6"/>
+    <mergeCell ref="AT6:AU6"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="AP6:AQ6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="AJ6:AK6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AD6:AE6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="G6:H6"/>
   </mergeCells>
   <conditionalFormatting sqref="D1:D1048576 F1:F1048576 H1:H1048576 J1:J1048576 L1:L1048576 N1:N1048576 Q1:Q1048576 S1:S1048576 U1:U1048576 W1:W1048576 Y1:Y1048576 AA1:AA1048576 AC1:AC1048576 AE1:AE1048576 AG1:AG1048576 AI1:AI1048576 AK1:AK1048576 AM1:AM1048576 AO1:AO1048576 AQ1:AQ1048576 AS1:AS1048576 AU1:AU1048576 AW1:AW1048576 AY1:AY1048576 BA1:BA1048576 BC1:BC1048576 BE1:BE1048576 BG1:BG1048576 BI1:BI1048576 BK1:BK1048576 BM1:BM1048576 BO1:BO1048576 BQ1:BQ1048576">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">

</xml_diff>

<commit_message>
Move test panel styling to XAML and declare shared style sources
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
+++ b/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\tests\PersonalEventBuilder\Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33261F51-14A9-4980-938D-C463F45BDFB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90C40287-E56F-411F-AA32-ECE97DC6D80B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -636,7 +636,7 @@
     <t>м. Тестоград</t>
   </si>
   <si>
-    <t>Щорічна відпустка</t>
+    <t>Відпустка за сімейними обставинами</t>
   </si>
 </sst>
 </file>
@@ -2268,125 +2268,125 @@
     <xf numFmtId="164" fontId="38" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="161">
@@ -4034,7 +4034,7 @@
       <c r="P8" s="65"/>
       <c r="Q8" s="56"/>
     </row>
-    <row r="9" spans="1:17" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A9" s="76"/>
       <c r="B9" s="77" t="s">
         <v>168</v>
@@ -4075,7 +4075,7 @@
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B9">
-    <cfRule type="duplicateValues" dxfId="2" priority="20784"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="20789"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -4177,311 +4177,311 @@
     </row>
     <row r="3" spans="1:69" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="109" t="s">
+      <c r="A4" s="103" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="117"/>
-      <c r="C4" s="109" t="s">
+      <c r="B4" s="111"/>
+      <c r="C4" s="103" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="118"/>
-      <c r="E4" s="118"/>
-      <c r="F4" s="118"/>
-      <c r="G4" s="118"/>
-      <c r="H4" s="119"/>
-      <c r="I4" s="96" t="s">
+      <c r="D4" s="115"/>
+      <c r="E4" s="115"/>
+      <c r="F4" s="115"/>
+      <c r="G4" s="115"/>
+      <c r="H4" s="116"/>
+      <c r="I4" s="90" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="97"/>
-      <c r="K4" s="98"/>
-      <c r="L4" s="99"/>
-      <c r="M4" s="99"/>
-      <c r="N4" s="100"/>
-      <c r="O4" s="124" t="s">
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
+      <c r="L4" s="93"/>
+      <c r="M4" s="93"/>
+      <c r="N4" s="94"/>
+      <c r="O4" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="P4" s="123" t="s">
+      <c r="P4" s="120" t="s">
         <v>24</v>
       </c>
-      <c r="Q4" s="124"/>
-      <c r="R4" s="124"/>
-      <c r="S4" s="124"/>
-      <c r="T4" s="124"/>
-      <c r="U4" s="125"/>
-      <c r="V4" s="106" t="s">
+      <c r="Q4" s="121"/>
+      <c r="R4" s="121"/>
+      <c r="S4" s="121"/>
+      <c r="T4" s="121"/>
+      <c r="U4" s="122"/>
+      <c r="V4" s="100" t="s">
         <v>25</v>
       </c>
-      <c r="W4" s="107"/>
-      <c r="X4" s="107"/>
-      <c r="Y4" s="107"/>
-      <c r="Z4" s="107"/>
-      <c r="AA4" s="107"/>
-      <c r="AB4" s="107"/>
-      <c r="AC4" s="107"/>
-      <c r="AD4" s="107"/>
-      <c r="AE4" s="107"/>
-      <c r="AF4" s="107"/>
-      <c r="AG4" s="107"/>
-      <c r="AH4" s="107"/>
-      <c r="AI4" s="107"/>
-      <c r="AJ4" s="107"/>
-      <c r="AK4" s="107"/>
-      <c r="AL4" s="107"/>
-      <c r="AM4" s="107"/>
-      <c r="AN4" s="107"/>
-      <c r="AO4" s="107"/>
-      <c r="AP4" s="107"/>
-      <c r="AQ4" s="107"/>
-      <c r="AR4" s="107"/>
-      <c r="AS4" s="107"/>
-      <c r="AT4" s="107"/>
-      <c r="AU4" s="107"/>
-      <c r="AV4" s="107"/>
-      <c r="AW4" s="107"/>
-      <c r="AX4" s="107"/>
-      <c r="AY4" s="107"/>
-      <c r="AZ4" s="107"/>
-      <c r="BA4" s="107"/>
-      <c r="BB4" s="107"/>
-      <c r="BC4" s="107"/>
-      <c r="BD4" s="107"/>
-      <c r="BE4" s="107"/>
-      <c r="BF4" s="107"/>
-      <c r="BG4" s="107"/>
-      <c r="BH4" s="107"/>
-      <c r="BI4" s="107"/>
-      <c r="BJ4" s="107"/>
-      <c r="BK4" s="107"/>
-      <c r="BL4" s="107"/>
-      <c r="BM4" s="107"/>
-      <c r="BN4" s="107"/>
-      <c r="BO4" s="107"/>
-      <c r="BP4" s="107"/>
-      <c r="BQ4" s="108"/>
+      <c r="W4" s="101"/>
+      <c r="X4" s="101"/>
+      <c r="Y4" s="101"/>
+      <c r="Z4" s="101"/>
+      <c r="AA4" s="101"/>
+      <c r="AB4" s="101"/>
+      <c r="AC4" s="101"/>
+      <c r="AD4" s="101"/>
+      <c r="AE4" s="101"/>
+      <c r="AF4" s="101"/>
+      <c r="AG4" s="101"/>
+      <c r="AH4" s="101"/>
+      <c r="AI4" s="101"/>
+      <c r="AJ4" s="101"/>
+      <c r="AK4" s="101"/>
+      <c r="AL4" s="101"/>
+      <c r="AM4" s="101"/>
+      <c r="AN4" s="101"/>
+      <c r="AO4" s="101"/>
+      <c r="AP4" s="101"/>
+      <c r="AQ4" s="101"/>
+      <c r="AR4" s="101"/>
+      <c r="AS4" s="101"/>
+      <c r="AT4" s="101"/>
+      <c r="AU4" s="101"/>
+      <c r="AV4" s="101"/>
+      <c r="AW4" s="101"/>
+      <c r="AX4" s="101"/>
+      <c r="AY4" s="101"/>
+      <c r="AZ4" s="101"/>
+      <c r="BA4" s="101"/>
+      <c r="BB4" s="101"/>
+      <c r="BC4" s="101"/>
+      <c r="BD4" s="101"/>
+      <c r="BE4" s="101"/>
+      <c r="BF4" s="101"/>
+      <c r="BG4" s="101"/>
+      <c r="BH4" s="101"/>
+      <c r="BI4" s="101"/>
+      <c r="BJ4" s="101"/>
+      <c r="BK4" s="101"/>
+      <c r="BL4" s="101"/>
+      <c r="BM4" s="101"/>
+      <c r="BN4" s="101"/>
+      <c r="BO4" s="101"/>
+      <c r="BP4" s="101"/>
+      <c r="BQ4" s="102"/>
     </row>
     <row r="5" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="110"/>
-      <c r="B5" s="117"/>
-      <c r="C5" s="120"/>
-      <c r="D5" s="121"/>
-      <c r="E5" s="121"/>
-      <c r="F5" s="121"/>
-      <c r="G5" s="121"/>
-      <c r="H5" s="122"/>
-      <c r="I5" s="101"/>
-      <c r="J5" s="102"/>
-      <c r="K5" s="103"/>
-      <c r="L5" s="104"/>
-      <c r="M5" s="104"/>
-      <c r="N5" s="105"/>
-      <c r="O5" s="129"/>
-      <c r="P5" s="126"/>
-      <c r="Q5" s="127"/>
-      <c r="R5" s="127"/>
-      <c r="S5" s="127"/>
-      <c r="T5" s="127"/>
-      <c r="U5" s="128"/>
-      <c r="V5" s="111" t="s">
+      <c r="A5" s="104"/>
+      <c r="B5" s="111"/>
+      <c r="C5" s="117"/>
+      <c r="D5" s="118"/>
+      <c r="E5" s="118"/>
+      <c r="F5" s="118"/>
+      <c r="G5" s="118"/>
+      <c r="H5" s="119"/>
+      <c r="I5" s="95"/>
+      <c r="J5" s="96"/>
+      <c r="K5" s="97"/>
+      <c r="L5" s="98"/>
+      <c r="M5" s="98"/>
+      <c r="N5" s="99"/>
+      <c r="O5" s="126"/>
+      <c r="P5" s="123"/>
+      <c r="Q5" s="124"/>
+      <c r="R5" s="124"/>
+      <c r="S5" s="124"/>
+      <c r="T5" s="124"/>
+      <c r="U5" s="125"/>
+      <c r="V5" s="105" t="s">
         <v>19</v>
       </c>
-      <c r="W5" s="112"/>
-      <c r="X5" s="112"/>
-      <c r="Y5" s="112"/>
-      <c r="Z5" s="112"/>
-      <c r="AA5" s="113"/>
-      <c r="AB5" s="114" t="s">
+      <c r="W5" s="106"/>
+      <c r="X5" s="106"/>
+      <c r="Y5" s="106"/>
+      <c r="Z5" s="106"/>
+      <c r="AA5" s="107"/>
+      <c r="AB5" s="108" t="s">
         <v>18</v>
       </c>
-      <c r="AC5" s="115"/>
-      <c r="AD5" s="115"/>
-      <c r="AE5" s="115"/>
-      <c r="AF5" s="115"/>
-      <c r="AG5" s="116"/>
-      <c r="AH5" s="114" t="s">
+      <c r="AC5" s="109"/>
+      <c r="AD5" s="109"/>
+      <c r="AE5" s="109"/>
+      <c r="AF5" s="109"/>
+      <c r="AG5" s="110"/>
+      <c r="AH5" s="108" t="s">
         <v>26</v>
       </c>
-      <c r="AI5" s="115"/>
-      <c r="AJ5" s="115"/>
-      <c r="AK5" s="115"/>
-      <c r="AL5" s="115"/>
-      <c r="AM5" s="116"/>
-      <c r="AN5" s="114" t="s">
+      <c r="AI5" s="109"/>
+      <c r="AJ5" s="109"/>
+      <c r="AK5" s="109"/>
+      <c r="AL5" s="109"/>
+      <c r="AM5" s="110"/>
+      <c r="AN5" s="108" t="s">
         <v>27</v>
       </c>
-      <c r="AO5" s="115"/>
-      <c r="AP5" s="115"/>
-      <c r="AQ5" s="115"/>
-      <c r="AR5" s="115"/>
-      <c r="AS5" s="116"/>
-      <c r="AT5" s="114" t="s">
+      <c r="AO5" s="109"/>
+      <c r="AP5" s="109"/>
+      <c r="AQ5" s="109"/>
+      <c r="AR5" s="109"/>
+      <c r="AS5" s="110"/>
+      <c r="AT5" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="AU5" s="115"/>
-      <c r="AV5" s="115"/>
-      <c r="AW5" s="115"/>
-      <c r="AX5" s="115"/>
-      <c r="AY5" s="116"/>
-      <c r="AZ5" s="114" t="s">
+      <c r="AU5" s="109"/>
+      <c r="AV5" s="109"/>
+      <c r="AW5" s="109"/>
+      <c r="AX5" s="109"/>
+      <c r="AY5" s="110"/>
+      <c r="AZ5" s="108" t="s">
         <v>29</v>
       </c>
-      <c r="BA5" s="115"/>
-      <c r="BB5" s="115"/>
-      <c r="BC5" s="115"/>
-      <c r="BD5" s="115"/>
-      <c r="BE5" s="116"/>
-      <c r="BF5" s="114" t="s">
+      <c r="BA5" s="109"/>
+      <c r="BB5" s="109"/>
+      <c r="BC5" s="109"/>
+      <c r="BD5" s="109"/>
+      <c r="BE5" s="110"/>
+      <c r="BF5" s="108" t="s">
         <v>30</v>
       </c>
-      <c r="BG5" s="115"/>
-      <c r="BH5" s="115"/>
-      <c r="BI5" s="115"/>
-      <c r="BJ5" s="115"/>
-      <c r="BK5" s="116"/>
-      <c r="BL5" s="96" t="s">
+      <c r="BG5" s="109"/>
+      <c r="BH5" s="109"/>
+      <c r="BI5" s="109"/>
+      <c r="BJ5" s="109"/>
+      <c r="BK5" s="110"/>
+      <c r="BL5" s="90" t="s">
         <v>31</v>
       </c>
-      <c r="BM5" s="98"/>
-      <c r="BN5" s="98"/>
-      <c r="BO5" s="99"/>
-      <c r="BP5" s="99"/>
-      <c r="BQ5" s="100"/>
+      <c r="BM5" s="92"/>
+      <c r="BN5" s="92"/>
+      <c r="BO5" s="93"/>
+      <c r="BP5" s="93"/>
+      <c r="BQ5" s="94"/>
     </row>
     <row r="6" spans="1:69" ht="103.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="110"/>
-      <c r="B6" s="95"/>
-      <c r="C6" s="90" t="s">
+      <c r="A6" s="104"/>
+      <c r="B6" s="112"/>
+      <c r="C6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="91"/>
-      <c r="E6" s="90" t="s">
+      <c r="D6" s="129"/>
+      <c r="E6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="91"/>
-      <c r="G6" s="90" t="s">
+      <c r="F6" s="129"/>
+      <c r="G6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="91"/>
-      <c r="I6" s="90" t="s">
+      <c r="H6" s="129"/>
+      <c r="I6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="J6" s="91"/>
-      <c r="K6" s="90" t="s">
+      <c r="J6" s="129"/>
+      <c r="K6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="L6" s="91"/>
-      <c r="M6" s="90" t="s">
+      <c r="L6" s="129"/>
+      <c r="M6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="N6" s="91"/>
-      <c r="O6" s="127"/>
-      <c r="P6" s="90" t="s">
+      <c r="N6" s="129"/>
+      <c r="O6" s="124"/>
+      <c r="P6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="Q6" s="91"/>
-      <c r="R6" s="90" t="s">
+      <c r="Q6" s="129"/>
+      <c r="R6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="S6" s="91"/>
-      <c r="T6" s="90" t="s">
+      <c r="S6" s="129"/>
+      <c r="T6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="U6" s="91"/>
-      <c r="V6" s="95" t="s">
+      <c r="U6" s="129"/>
+      <c r="V6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="W6" s="94"/>
-      <c r="X6" s="92" t="s">
+      <c r="W6" s="127"/>
+      <c r="X6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="Y6" s="94"/>
-      <c r="Z6" s="92" t="s">
+      <c r="Y6" s="127"/>
+      <c r="Z6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AA6" s="93"/>
-      <c r="AB6" s="95" t="s">
+      <c r="AA6" s="114"/>
+      <c r="AB6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AC6" s="94"/>
-      <c r="AD6" s="92" t="s">
+      <c r="AC6" s="127"/>
+      <c r="AD6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AE6" s="94"/>
-      <c r="AF6" s="92" t="s">
+      <c r="AE6" s="127"/>
+      <c r="AF6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AG6" s="93"/>
-      <c r="AH6" s="95" t="s">
+      <c r="AG6" s="114"/>
+      <c r="AH6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AI6" s="94"/>
-      <c r="AJ6" s="92" t="s">
+      <c r="AI6" s="127"/>
+      <c r="AJ6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AK6" s="94"/>
-      <c r="AL6" s="92" t="s">
+      <c r="AK6" s="127"/>
+      <c r="AL6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AM6" s="93"/>
-      <c r="AN6" s="95" t="s">
+      <c r="AM6" s="114"/>
+      <c r="AN6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AO6" s="94"/>
-      <c r="AP6" s="92" t="s">
+      <c r="AO6" s="127"/>
+      <c r="AP6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AQ6" s="94"/>
-      <c r="AR6" s="92" t="s">
+      <c r="AQ6" s="127"/>
+      <c r="AR6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AS6" s="93"/>
-      <c r="AT6" s="95" t="s">
+      <c r="AS6" s="114"/>
+      <c r="AT6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AU6" s="94"/>
-      <c r="AV6" s="92" t="s">
+      <c r="AU6" s="127"/>
+      <c r="AV6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AW6" s="94"/>
-      <c r="AX6" s="92" t="s">
+      <c r="AW6" s="127"/>
+      <c r="AX6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AY6" s="93"/>
-      <c r="AZ6" s="95" t="s">
+      <c r="AY6" s="114"/>
+      <c r="AZ6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BA6" s="94"/>
-      <c r="BB6" s="92" t="s">
+      <c r="BA6" s="127"/>
+      <c r="BB6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BC6" s="94"/>
-      <c r="BD6" s="92" t="s">
+      <c r="BC6" s="127"/>
+      <c r="BD6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BE6" s="93"/>
-      <c r="BF6" s="95" t="s">
+      <c r="BE6" s="114"/>
+      <c r="BF6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BG6" s="94"/>
-      <c r="BH6" s="92" t="s">
+      <c r="BG6" s="127"/>
+      <c r="BH6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BI6" s="94"/>
-      <c r="BJ6" s="92" t="s">
+      <c r="BI6" s="127"/>
+      <c r="BJ6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BK6" s="93"/>
-      <c r="BL6" s="95" t="s">
+      <c r="BK6" s="114"/>
+      <c r="BL6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BM6" s="94"/>
-      <c r="BN6" s="92" t="s">
+      <c r="BM6" s="127"/>
+      <c r="BN6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BO6" s="94"/>
-      <c r="BP6" s="92" t="s">
+      <c r="BO6" s="127"/>
+      <c r="BP6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BQ6" s="93"/>
+      <c r="BQ6" s="114"/>
     </row>
     <row r="7" spans="1:69" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
@@ -10552,6 +10552,38 @@
     </row>
   </sheetData>
   <mergeCells count="48">
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="AJ6:AK6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AD6:AE6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AT6:AU6"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="AP6:AQ6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="BD6:BE6"/>
+    <mergeCell ref="BB6:BC6"/>
+    <mergeCell ref="AZ6:BA6"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AV6:AW6"/>
+    <mergeCell ref="BN6:BO6"/>
+    <mergeCell ref="BL6:BM6"/>
+    <mergeCell ref="BJ6:BK6"/>
+    <mergeCell ref="BH6:BI6"/>
+    <mergeCell ref="BF6:BG6"/>
     <mergeCell ref="I4:N5"/>
     <mergeCell ref="V4:BQ4"/>
     <mergeCell ref="A4:A6"/>
@@ -10568,38 +10600,6 @@
     <mergeCell ref="C4:H5"/>
     <mergeCell ref="P4:U5"/>
     <mergeCell ref="O4:O6"/>
-    <mergeCell ref="BN6:BO6"/>
-    <mergeCell ref="BL6:BM6"/>
-    <mergeCell ref="BJ6:BK6"/>
-    <mergeCell ref="BH6:BI6"/>
-    <mergeCell ref="BF6:BG6"/>
-    <mergeCell ref="BD6:BE6"/>
-    <mergeCell ref="BB6:BC6"/>
-    <mergeCell ref="AZ6:BA6"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AV6:AW6"/>
-    <mergeCell ref="AT6:AU6"/>
-    <mergeCell ref="AR6:AS6"/>
-    <mergeCell ref="AP6:AQ6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="AJ6:AK6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AD6:AE6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="X6:Y6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="R6:S6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="G6:H6"/>
   </mergeCells>
   <conditionalFormatting sqref="D1:D1048576 F1:F1048576 H1:H1048576 J1:J1048576 L1:L1048576 N1:N1048576 Q1:Q1048576 S1:S1048576 U1:U1048576 W1:W1048576 Y1:Y1048576 AA1:AA1048576 AC1:AC1048576 AE1:AE1048576 AG1:AG1048576 AI1:AI1048576 AK1:AK1048576 AM1:AM1048576 AO1:AO1048576 AQ1:AQ1048576 AS1:AS1048576 AU1:AU1048576 AW1:AW1048576 AY1:AY1048576 BA1:BA1048576 BC1:BC1048576 BE1:BE1048576 BG1:BG1048576 BI1:BI1048576 BK1:BK1048576 BM1:BM1048576 BO1:BO1048576 BQ1:BQ1048576">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">

</xml_diff>

<commit_message>
Optimize PEB test execution and add per-scenario preview controls
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
+++ b/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\tests\PersonalEventBuilder\Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90C40287-E56F-411F-AA32-ECE97DC6D80B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F34EDD-E2E3-434B-93F5-5EB493875251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
     <definedName name="_Hlk209437159" localSheetId="0">'5. Тимчасово відсутні'!#REF!</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Т (Х)'!$A$1:$BQ$30</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcMode="manual"/>
+  <calcPr calcId="191029" calcMode="manual" calcCompleted="0" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2268,6 +2268,24 @@
     <xf numFmtId="164" fontId="38" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2334,15 +2352,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2378,15 +2387,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="161">
@@ -4075,7 +4075,7 @@
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B9">
-    <cfRule type="duplicateValues" dxfId="2" priority="20789"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="20798"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -4177,311 +4177,311 @@
     </row>
     <row r="3" spans="1:69" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="103" t="s">
+      <c r="A4" s="109" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="111"/>
-      <c r="C4" s="103" t="s">
+      <c r="B4" s="117"/>
+      <c r="C4" s="109" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="115"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="116"/>
-      <c r="I4" s="90" t="s">
+      <c r="D4" s="118"/>
+      <c r="E4" s="118"/>
+      <c r="F4" s="118"/>
+      <c r="G4" s="118"/>
+      <c r="H4" s="119"/>
+      <c r="I4" s="96" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
-      <c r="L4" s="93"/>
-      <c r="M4" s="93"/>
-      <c r="N4" s="94"/>
-      <c r="O4" s="121" t="s">
+      <c r="J4" s="97"/>
+      <c r="K4" s="98"/>
+      <c r="L4" s="99"/>
+      <c r="M4" s="99"/>
+      <c r="N4" s="100"/>
+      <c r="O4" s="124" t="s">
         <v>23</v>
       </c>
-      <c r="P4" s="120" t="s">
+      <c r="P4" s="123" t="s">
         <v>24</v>
       </c>
-      <c r="Q4" s="121"/>
-      <c r="R4" s="121"/>
-      <c r="S4" s="121"/>
-      <c r="T4" s="121"/>
-      <c r="U4" s="122"/>
-      <c r="V4" s="100" t="s">
+      <c r="Q4" s="124"/>
+      <c r="R4" s="124"/>
+      <c r="S4" s="124"/>
+      <c r="T4" s="124"/>
+      <c r="U4" s="125"/>
+      <c r="V4" s="106" t="s">
         <v>25</v>
       </c>
-      <c r="W4" s="101"/>
-      <c r="X4" s="101"/>
-      <c r="Y4" s="101"/>
-      <c r="Z4" s="101"/>
-      <c r="AA4" s="101"/>
-      <c r="AB4" s="101"/>
-      <c r="AC4" s="101"/>
-      <c r="AD4" s="101"/>
-      <c r="AE4" s="101"/>
-      <c r="AF4" s="101"/>
-      <c r="AG4" s="101"/>
-      <c r="AH4" s="101"/>
-      <c r="AI4" s="101"/>
-      <c r="AJ4" s="101"/>
-      <c r="AK4" s="101"/>
-      <c r="AL4" s="101"/>
-      <c r="AM4" s="101"/>
-      <c r="AN4" s="101"/>
-      <c r="AO4" s="101"/>
-      <c r="AP4" s="101"/>
-      <c r="AQ4" s="101"/>
-      <c r="AR4" s="101"/>
-      <c r="AS4" s="101"/>
-      <c r="AT4" s="101"/>
-      <c r="AU4" s="101"/>
-      <c r="AV4" s="101"/>
-      <c r="AW4" s="101"/>
-      <c r="AX4" s="101"/>
-      <c r="AY4" s="101"/>
-      <c r="AZ4" s="101"/>
-      <c r="BA4" s="101"/>
-      <c r="BB4" s="101"/>
-      <c r="BC4" s="101"/>
-      <c r="BD4" s="101"/>
-      <c r="BE4" s="101"/>
-      <c r="BF4" s="101"/>
-      <c r="BG4" s="101"/>
-      <c r="BH4" s="101"/>
-      <c r="BI4" s="101"/>
-      <c r="BJ4" s="101"/>
-      <c r="BK4" s="101"/>
-      <c r="BL4" s="101"/>
-      <c r="BM4" s="101"/>
-      <c r="BN4" s="101"/>
-      <c r="BO4" s="101"/>
-      <c r="BP4" s="101"/>
-      <c r="BQ4" s="102"/>
+      <c r="W4" s="107"/>
+      <c r="X4" s="107"/>
+      <c r="Y4" s="107"/>
+      <c r="Z4" s="107"/>
+      <c r="AA4" s="107"/>
+      <c r="AB4" s="107"/>
+      <c r="AC4" s="107"/>
+      <c r="AD4" s="107"/>
+      <c r="AE4" s="107"/>
+      <c r="AF4" s="107"/>
+      <c r="AG4" s="107"/>
+      <c r="AH4" s="107"/>
+      <c r="AI4" s="107"/>
+      <c r="AJ4" s="107"/>
+      <c r="AK4" s="107"/>
+      <c r="AL4" s="107"/>
+      <c r="AM4" s="107"/>
+      <c r="AN4" s="107"/>
+      <c r="AO4" s="107"/>
+      <c r="AP4" s="107"/>
+      <c r="AQ4" s="107"/>
+      <c r="AR4" s="107"/>
+      <c r="AS4" s="107"/>
+      <c r="AT4" s="107"/>
+      <c r="AU4" s="107"/>
+      <c r="AV4" s="107"/>
+      <c r="AW4" s="107"/>
+      <c r="AX4" s="107"/>
+      <c r="AY4" s="107"/>
+      <c r="AZ4" s="107"/>
+      <c r="BA4" s="107"/>
+      <c r="BB4" s="107"/>
+      <c r="BC4" s="107"/>
+      <c r="BD4" s="107"/>
+      <c r="BE4" s="107"/>
+      <c r="BF4" s="107"/>
+      <c r="BG4" s="107"/>
+      <c r="BH4" s="107"/>
+      <c r="BI4" s="107"/>
+      <c r="BJ4" s="107"/>
+      <c r="BK4" s="107"/>
+      <c r="BL4" s="107"/>
+      <c r="BM4" s="107"/>
+      <c r="BN4" s="107"/>
+      <c r="BO4" s="107"/>
+      <c r="BP4" s="107"/>
+      <c r="BQ4" s="108"/>
     </row>
     <row r="5" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="104"/>
-      <c r="B5" s="111"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="118"/>
-      <c r="E5" s="118"/>
-      <c r="F5" s="118"/>
-      <c r="G5" s="118"/>
-      <c r="H5" s="119"/>
-      <c r="I5" s="95"/>
-      <c r="J5" s="96"/>
-      <c r="K5" s="97"/>
-      <c r="L5" s="98"/>
-      <c r="M5" s="98"/>
-      <c r="N5" s="99"/>
-      <c r="O5" s="126"/>
-      <c r="P5" s="123"/>
-      <c r="Q5" s="124"/>
-      <c r="R5" s="124"/>
-      <c r="S5" s="124"/>
-      <c r="T5" s="124"/>
-      <c r="U5" s="125"/>
-      <c r="V5" s="105" t="s">
+      <c r="A5" s="110"/>
+      <c r="B5" s="117"/>
+      <c r="C5" s="120"/>
+      <c r="D5" s="121"/>
+      <c r="E5" s="121"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="121"/>
+      <c r="H5" s="122"/>
+      <c r="I5" s="101"/>
+      <c r="J5" s="102"/>
+      <c r="K5" s="103"/>
+      <c r="L5" s="104"/>
+      <c r="M5" s="104"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="129"/>
+      <c r="P5" s="126"/>
+      <c r="Q5" s="127"/>
+      <c r="R5" s="127"/>
+      <c r="S5" s="127"/>
+      <c r="T5" s="127"/>
+      <c r="U5" s="128"/>
+      <c r="V5" s="111" t="s">
         <v>19</v>
       </c>
-      <c r="W5" s="106"/>
-      <c r="X5" s="106"/>
-      <c r="Y5" s="106"/>
-      <c r="Z5" s="106"/>
-      <c r="AA5" s="107"/>
-      <c r="AB5" s="108" t="s">
+      <c r="W5" s="112"/>
+      <c r="X5" s="112"/>
+      <c r="Y5" s="112"/>
+      <c r="Z5" s="112"/>
+      <c r="AA5" s="113"/>
+      <c r="AB5" s="114" t="s">
         <v>18</v>
       </c>
-      <c r="AC5" s="109"/>
-      <c r="AD5" s="109"/>
-      <c r="AE5" s="109"/>
-      <c r="AF5" s="109"/>
-      <c r="AG5" s="110"/>
-      <c r="AH5" s="108" t="s">
+      <c r="AC5" s="115"/>
+      <c r="AD5" s="115"/>
+      <c r="AE5" s="115"/>
+      <c r="AF5" s="115"/>
+      <c r="AG5" s="116"/>
+      <c r="AH5" s="114" t="s">
         <v>26</v>
       </c>
-      <c r="AI5" s="109"/>
-      <c r="AJ5" s="109"/>
-      <c r="AK5" s="109"/>
-      <c r="AL5" s="109"/>
-      <c r="AM5" s="110"/>
-      <c r="AN5" s="108" t="s">
+      <c r="AI5" s="115"/>
+      <c r="AJ5" s="115"/>
+      <c r="AK5" s="115"/>
+      <c r="AL5" s="115"/>
+      <c r="AM5" s="116"/>
+      <c r="AN5" s="114" t="s">
         <v>27</v>
       </c>
-      <c r="AO5" s="109"/>
-      <c r="AP5" s="109"/>
-      <c r="AQ5" s="109"/>
-      <c r="AR5" s="109"/>
-      <c r="AS5" s="110"/>
-      <c r="AT5" s="108" t="s">
+      <c r="AO5" s="115"/>
+      <c r="AP5" s="115"/>
+      <c r="AQ5" s="115"/>
+      <c r="AR5" s="115"/>
+      <c r="AS5" s="116"/>
+      <c r="AT5" s="114" t="s">
         <v>28</v>
       </c>
-      <c r="AU5" s="109"/>
-      <c r="AV5" s="109"/>
-      <c r="AW5" s="109"/>
-      <c r="AX5" s="109"/>
-      <c r="AY5" s="110"/>
-      <c r="AZ5" s="108" t="s">
+      <c r="AU5" s="115"/>
+      <c r="AV5" s="115"/>
+      <c r="AW5" s="115"/>
+      <c r="AX5" s="115"/>
+      <c r="AY5" s="116"/>
+      <c r="AZ5" s="114" t="s">
         <v>29</v>
       </c>
-      <c r="BA5" s="109"/>
-      <c r="BB5" s="109"/>
-      <c r="BC5" s="109"/>
-      <c r="BD5" s="109"/>
-      <c r="BE5" s="110"/>
-      <c r="BF5" s="108" t="s">
+      <c r="BA5" s="115"/>
+      <c r="BB5" s="115"/>
+      <c r="BC5" s="115"/>
+      <c r="BD5" s="115"/>
+      <c r="BE5" s="116"/>
+      <c r="BF5" s="114" t="s">
         <v>30</v>
       </c>
-      <c r="BG5" s="109"/>
-      <c r="BH5" s="109"/>
-      <c r="BI5" s="109"/>
-      <c r="BJ5" s="109"/>
-      <c r="BK5" s="110"/>
-      <c r="BL5" s="90" t="s">
+      <c r="BG5" s="115"/>
+      <c r="BH5" s="115"/>
+      <c r="BI5" s="115"/>
+      <c r="BJ5" s="115"/>
+      <c r="BK5" s="116"/>
+      <c r="BL5" s="96" t="s">
         <v>31</v>
       </c>
-      <c r="BM5" s="92"/>
-      <c r="BN5" s="92"/>
-      <c r="BO5" s="93"/>
-      <c r="BP5" s="93"/>
-      <c r="BQ5" s="94"/>
+      <c r="BM5" s="98"/>
+      <c r="BN5" s="98"/>
+      <c r="BO5" s="99"/>
+      <c r="BP5" s="99"/>
+      <c r="BQ5" s="100"/>
     </row>
     <row r="6" spans="1:69" ht="103.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="104"/>
-      <c r="B6" s="112"/>
-      <c r="C6" s="128" t="s">
+      <c r="A6" s="110"/>
+      <c r="B6" s="95"/>
+      <c r="C6" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="129"/>
-      <c r="E6" s="128" t="s">
+      <c r="D6" s="91"/>
+      <c r="E6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="129"/>
-      <c r="G6" s="128" t="s">
+      <c r="F6" s="91"/>
+      <c r="G6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="129"/>
-      <c r="I6" s="128" t="s">
+      <c r="H6" s="91"/>
+      <c r="I6" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="J6" s="129"/>
-      <c r="K6" s="128" t="s">
+      <c r="J6" s="91"/>
+      <c r="K6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="L6" s="129"/>
-      <c r="M6" s="128" t="s">
+      <c r="L6" s="91"/>
+      <c r="M6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="N6" s="129"/>
-      <c r="O6" s="124"/>
-      <c r="P6" s="128" t="s">
+      <c r="N6" s="91"/>
+      <c r="O6" s="127"/>
+      <c r="P6" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="Q6" s="129"/>
-      <c r="R6" s="128" t="s">
+      <c r="Q6" s="91"/>
+      <c r="R6" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="S6" s="129"/>
-      <c r="T6" s="128" t="s">
+      <c r="S6" s="91"/>
+      <c r="T6" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="U6" s="129"/>
-      <c r="V6" s="112" t="s">
+      <c r="U6" s="91"/>
+      <c r="V6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="W6" s="127"/>
-      <c r="X6" s="113" t="s">
+      <c r="W6" s="94"/>
+      <c r="X6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="Y6" s="127"/>
-      <c r="Z6" s="113" t="s">
+      <c r="Y6" s="94"/>
+      <c r="Z6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AA6" s="114"/>
-      <c r="AB6" s="112" t="s">
+      <c r="AA6" s="93"/>
+      <c r="AB6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AC6" s="127"/>
-      <c r="AD6" s="113" t="s">
+      <c r="AC6" s="94"/>
+      <c r="AD6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AE6" s="127"/>
-      <c r="AF6" s="113" t="s">
+      <c r="AE6" s="94"/>
+      <c r="AF6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AG6" s="114"/>
-      <c r="AH6" s="112" t="s">
+      <c r="AG6" s="93"/>
+      <c r="AH6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AI6" s="127"/>
-      <c r="AJ6" s="113" t="s">
+      <c r="AI6" s="94"/>
+      <c r="AJ6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AK6" s="127"/>
-      <c r="AL6" s="113" t="s">
+      <c r="AK6" s="94"/>
+      <c r="AL6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AM6" s="114"/>
-      <c r="AN6" s="112" t="s">
+      <c r="AM6" s="93"/>
+      <c r="AN6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AO6" s="127"/>
-      <c r="AP6" s="113" t="s">
+      <c r="AO6" s="94"/>
+      <c r="AP6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AQ6" s="127"/>
-      <c r="AR6" s="113" t="s">
+      <c r="AQ6" s="94"/>
+      <c r="AR6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AS6" s="114"/>
-      <c r="AT6" s="112" t="s">
+      <c r="AS6" s="93"/>
+      <c r="AT6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="AU6" s="127"/>
-      <c r="AV6" s="113" t="s">
+      <c r="AU6" s="94"/>
+      <c r="AV6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="AW6" s="127"/>
-      <c r="AX6" s="113" t="s">
+      <c r="AW6" s="94"/>
+      <c r="AX6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AY6" s="114"/>
-      <c r="AZ6" s="112" t="s">
+      <c r="AY6" s="93"/>
+      <c r="AZ6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="BA6" s="127"/>
-      <c r="BB6" s="113" t="s">
+      <c r="BA6" s="94"/>
+      <c r="BB6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BC6" s="127"/>
-      <c r="BD6" s="113" t="s">
+      <c r="BC6" s="94"/>
+      <c r="BD6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BE6" s="114"/>
-      <c r="BF6" s="112" t="s">
+      <c r="BE6" s="93"/>
+      <c r="BF6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="BG6" s="127"/>
-      <c r="BH6" s="113" t="s">
+      <c r="BG6" s="94"/>
+      <c r="BH6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BI6" s="127"/>
-      <c r="BJ6" s="113" t="s">
+      <c r="BI6" s="94"/>
+      <c r="BJ6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BK6" s="114"/>
-      <c r="BL6" s="112" t="s">
+      <c r="BK6" s="93"/>
+      <c r="BL6" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="BM6" s="127"/>
-      <c r="BN6" s="113" t="s">
+      <c r="BM6" s="94"/>
+      <c r="BN6" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="BO6" s="127"/>
-      <c r="BP6" s="113" t="s">
+      <c r="BO6" s="94"/>
+      <c r="BP6" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="BQ6" s="114"/>
+      <c r="BQ6" s="93"/>
     </row>
     <row r="7" spans="1:69" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
@@ -10552,38 +10552,6 @@
     </row>
   </sheetData>
   <mergeCells count="48">
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="X6:Y6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="R6:S6"/>
-    <mergeCell ref="AJ6:AK6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AD6:AE6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AT6:AU6"/>
-    <mergeCell ref="AR6:AS6"/>
-    <mergeCell ref="AP6:AQ6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="BD6:BE6"/>
-    <mergeCell ref="BB6:BC6"/>
-    <mergeCell ref="AZ6:BA6"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AV6:AW6"/>
-    <mergeCell ref="BN6:BO6"/>
-    <mergeCell ref="BL6:BM6"/>
-    <mergeCell ref="BJ6:BK6"/>
-    <mergeCell ref="BH6:BI6"/>
-    <mergeCell ref="BF6:BG6"/>
     <mergeCell ref="I4:N5"/>
     <mergeCell ref="V4:BQ4"/>
     <mergeCell ref="A4:A6"/>
@@ -10600,6 +10568,38 @@
     <mergeCell ref="C4:H5"/>
     <mergeCell ref="P4:U5"/>
     <mergeCell ref="O4:O6"/>
+    <mergeCell ref="BN6:BO6"/>
+    <mergeCell ref="BL6:BM6"/>
+    <mergeCell ref="BJ6:BK6"/>
+    <mergeCell ref="BH6:BI6"/>
+    <mergeCell ref="BF6:BG6"/>
+    <mergeCell ref="BD6:BE6"/>
+    <mergeCell ref="BB6:BC6"/>
+    <mergeCell ref="AZ6:BA6"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AV6:AW6"/>
+    <mergeCell ref="AT6:AU6"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="AP6:AQ6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="AJ6:AK6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AD6:AE6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="G6:H6"/>
   </mergeCells>
   <conditionalFormatting sqref="D1:D1048576 F1:F1048576 H1:H1048576 J1:J1048576 L1:L1048576 N1:N1048576 Q1:Q1048576 S1:S1048576 U1:U1048576 W1:W1048576 Y1:Y1048576 AA1:AA1048576 AC1:AC1048576 AE1:AE1048576 AG1:AG1048576 AI1:AI1048576 AK1:AK1048576 AM1:AM1048576 AO1:AO1048576 AQ1:AQ1048576 AS1:AS1048576 AU1:AU1048576 AW1:AW1048576 AY1:AY1048576 BA1:BA1048576 BC1:BC1048576 BE1:BE1048576 BG1:BG1048576 BI1:BI1048576 BK1:BK1048576 BM1:BM1048576 BO1:BO1048576 BQ1:BQ1048576">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">

</xml_diff>

<commit_message>
Remove unsupported outpatient Word templates and fix VBA declarations
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
+++ b/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\tests\PersonalEventBuilder\Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F34EDD-E2E3-434B-93F5-5EB493875251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD0CC0B0-62A6-4776-B514-C7E2B86360CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -636,7 +636,7 @@
     <t>м. Тестоград</t>
   </si>
   <si>
-    <t>Відпустка за сімейними обставинами</t>
+    <t>Відпустка для лікування</t>
   </si>
 </sst>
 </file>
@@ -4075,7 +4075,7 @@
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B9">
-    <cfRule type="duplicateValues" dxfId="2" priority="20798"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="20801"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Add shared Word anchor testing and formatted test document output
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
+++ b/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\tests\PersonalEventBuilder\Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD0CC0B0-62A6-4776-B514-C7E2B86360CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0574ADC8-63D0-4BBB-9255-0B058AE2C51C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4075,7 +4075,7 @@
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B9">
-    <cfRule type="duplicateValues" dxfId="2" priority="20801"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="20816"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Update test worksheet references and move DSL checks to scripts
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
+++ b/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\tests\PersonalEventBuilder\Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0574ADC8-63D0-4BBB-9255-0B058AE2C51C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D687FA9E-468F-46EA-BA8F-755C48AAE456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -633,10 +633,10 @@
     <t>БОНДАРЕНКО Олександр Юрійович</t>
   </si>
   <si>
+    <t>Щорічна відпустка</t>
+  </si>
+  <si>
     <t>м. Тестоград</t>
-  </si>
-  <si>
-    <t>Відпустка для лікування</t>
   </si>
 </sst>
 </file>
@@ -2235,30 +2235,30 @@
     <xf numFmtId="0" fontId="43" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="43" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="45" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="46" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="43" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="44" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="43" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="45" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="46" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="43" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2268,125 +2268,125 @@
     <xf numFmtId="164" fontId="38" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="161">
@@ -4034,34 +4034,34 @@
       <c r="P8" s="65"/>
       <c r="Q8" s="56"/>
     </row>
-    <row r="9" spans="1:17" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A9" s="76"/>
       <c r="B9" s="77" t="s">
         <v>168</v>
       </c>
       <c r="C9" s="78"/>
-      <c r="D9" s="82" t="s">
+      <c r="D9" s="86" t="s">
+        <v>169</v>
+      </c>
+      <c r="E9" s="86" t="s">
         <v>170</v>
       </c>
-      <c r="E9" s="82" t="s">
-        <v>169</v>
-      </c>
-      <c r="F9" s="83">
+      <c r="F9" s="79">
         <v>46310</v>
       </c>
-      <c r="G9" s="83"/>
-      <c r="H9" s="83"/>
-      <c r="I9" s="79"/>
-      <c r="J9" s="84"/>
-      <c r="K9" s="83"/>
-      <c r="L9" s="83"/>
-      <c r="M9" s="83"/>
-      <c r="N9" s="80"/>
-      <c r="O9" s="81">
+      <c r="G9" s="79"/>
+      <c r="H9" s="79"/>
+      <c r="I9" s="80"/>
+      <c r="J9" s="81"/>
+      <c r="K9" s="79"/>
+      <c r="L9" s="79"/>
+      <c r="M9" s="79"/>
+      <c r="N9" s="82"/>
+      <c r="O9" s="83">
         <v>1</v>
       </c>
-      <c r="P9" s="85"/>
-      <c r="Q9" s="86"/>
+      <c r="P9" s="84"/>
+      <c r="Q9" s="85"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4075,7 +4075,7 @@
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B9">
-    <cfRule type="duplicateValues" dxfId="2" priority="20816"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="20823"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -4177,311 +4177,311 @@
     </row>
     <row r="3" spans="1:69" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="109" t="s">
+      <c r="A4" s="103" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="117"/>
-      <c r="C4" s="109" t="s">
+      <c r="B4" s="111"/>
+      <c r="C4" s="103" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="118"/>
-      <c r="E4" s="118"/>
-      <c r="F4" s="118"/>
-      <c r="G4" s="118"/>
-      <c r="H4" s="119"/>
-      <c r="I4" s="96" t="s">
+      <c r="D4" s="115"/>
+      <c r="E4" s="115"/>
+      <c r="F4" s="115"/>
+      <c r="G4" s="115"/>
+      <c r="H4" s="116"/>
+      <c r="I4" s="90" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="97"/>
-      <c r="K4" s="98"/>
-      <c r="L4" s="99"/>
-      <c r="M4" s="99"/>
-      <c r="N4" s="100"/>
-      <c r="O4" s="124" t="s">
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
+      <c r="L4" s="93"/>
+      <c r="M4" s="93"/>
+      <c r="N4" s="94"/>
+      <c r="O4" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="P4" s="123" t="s">
+      <c r="P4" s="120" t="s">
         <v>24</v>
       </c>
-      <c r="Q4" s="124"/>
-      <c r="R4" s="124"/>
-      <c r="S4" s="124"/>
-      <c r="T4" s="124"/>
-      <c r="U4" s="125"/>
-      <c r="V4" s="106" t="s">
+      <c r="Q4" s="121"/>
+      <c r="R4" s="121"/>
+      <c r="S4" s="121"/>
+      <c r="T4" s="121"/>
+      <c r="U4" s="122"/>
+      <c r="V4" s="100" t="s">
         <v>25</v>
       </c>
-      <c r="W4" s="107"/>
-      <c r="X4" s="107"/>
-      <c r="Y4" s="107"/>
-      <c r="Z4" s="107"/>
-      <c r="AA4" s="107"/>
-      <c r="AB4" s="107"/>
-      <c r="AC4" s="107"/>
-      <c r="AD4" s="107"/>
-      <c r="AE4" s="107"/>
-      <c r="AF4" s="107"/>
-      <c r="AG4" s="107"/>
-      <c r="AH4" s="107"/>
-      <c r="AI4" s="107"/>
-      <c r="AJ4" s="107"/>
-      <c r="AK4" s="107"/>
-      <c r="AL4" s="107"/>
-      <c r="AM4" s="107"/>
-      <c r="AN4" s="107"/>
-      <c r="AO4" s="107"/>
-      <c r="AP4" s="107"/>
-      <c r="AQ4" s="107"/>
-      <c r="AR4" s="107"/>
-      <c r="AS4" s="107"/>
-      <c r="AT4" s="107"/>
-      <c r="AU4" s="107"/>
-      <c r="AV4" s="107"/>
-      <c r="AW4" s="107"/>
-      <c r="AX4" s="107"/>
-      <c r="AY4" s="107"/>
-      <c r="AZ4" s="107"/>
-      <c r="BA4" s="107"/>
-      <c r="BB4" s="107"/>
-      <c r="BC4" s="107"/>
-      <c r="BD4" s="107"/>
-      <c r="BE4" s="107"/>
-      <c r="BF4" s="107"/>
-      <c r="BG4" s="107"/>
-      <c r="BH4" s="107"/>
-      <c r="BI4" s="107"/>
-      <c r="BJ4" s="107"/>
-      <c r="BK4" s="107"/>
-      <c r="BL4" s="107"/>
-      <c r="BM4" s="107"/>
-      <c r="BN4" s="107"/>
-      <c r="BO4" s="107"/>
-      <c r="BP4" s="107"/>
-      <c r="BQ4" s="108"/>
+      <c r="W4" s="101"/>
+      <c r="X4" s="101"/>
+      <c r="Y4" s="101"/>
+      <c r="Z4" s="101"/>
+      <c r="AA4" s="101"/>
+      <c r="AB4" s="101"/>
+      <c r="AC4" s="101"/>
+      <c r="AD4" s="101"/>
+      <c r="AE4" s="101"/>
+      <c r="AF4" s="101"/>
+      <c r="AG4" s="101"/>
+      <c r="AH4" s="101"/>
+      <c r="AI4" s="101"/>
+      <c r="AJ4" s="101"/>
+      <c r="AK4" s="101"/>
+      <c r="AL4" s="101"/>
+      <c r="AM4" s="101"/>
+      <c r="AN4" s="101"/>
+      <c r="AO4" s="101"/>
+      <c r="AP4" s="101"/>
+      <c r="AQ4" s="101"/>
+      <c r="AR4" s="101"/>
+      <c r="AS4" s="101"/>
+      <c r="AT4" s="101"/>
+      <c r="AU4" s="101"/>
+      <c r="AV4" s="101"/>
+      <c r="AW4" s="101"/>
+      <c r="AX4" s="101"/>
+      <c r="AY4" s="101"/>
+      <c r="AZ4" s="101"/>
+      <c r="BA4" s="101"/>
+      <c r="BB4" s="101"/>
+      <c r="BC4" s="101"/>
+      <c r="BD4" s="101"/>
+      <c r="BE4" s="101"/>
+      <c r="BF4" s="101"/>
+      <c r="BG4" s="101"/>
+      <c r="BH4" s="101"/>
+      <c r="BI4" s="101"/>
+      <c r="BJ4" s="101"/>
+      <c r="BK4" s="101"/>
+      <c r="BL4" s="101"/>
+      <c r="BM4" s="101"/>
+      <c r="BN4" s="101"/>
+      <c r="BO4" s="101"/>
+      <c r="BP4" s="101"/>
+      <c r="BQ4" s="102"/>
     </row>
     <row r="5" spans="1:69" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="110"/>
-      <c r="B5" s="117"/>
-      <c r="C5" s="120"/>
-      <c r="D5" s="121"/>
-      <c r="E5" s="121"/>
-      <c r="F5" s="121"/>
-      <c r="G5" s="121"/>
-      <c r="H5" s="122"/>
-      <c r="I5" s="101"/>
-      <c r="J5" s="102"/>
-      <c r="K5" s="103"/>
-      <c r="L5" s="104"/>
-      <c r="M5" s="104"/>
-      <c r="N5" s="105"/>
-      <c r="O5" s="129"/>
-      <c r="P5" s="126"/>
-      <c r="Q5" s="127"/>
-      <c r="R5" s="127"/>
-      <c r="S5" s="127"/>
-      <c r="T5" s="127"/>
-      <c r="U5" s="128"/>
-      <c r="V5" s="111" t="s">
+      <c r="A5" s="104"/>
+      <c r="B5" s="111"/>
+      <c r="C5" s="117"/>
+      <c r="D5" s="118"/>
+      <c r="E5" s="118"/>
+      <c r="F5" s="118"/>
+      <c r="G5" s="118"/>
+      <c r="H5" s="119"/>
+      <c r="I5" s="95"/>
+      <c r="J5" s="96"/>
+      <c r="K5" s="97"/>
+      <c r="L5" s="98"/>
+      <c r="M5" s="98"/>
+      <c r="N5" s="99"/>
+      <c r="O5" s="126"/>
+      <c r="P5" s="123"/>
+      <c r="Q5" s="124"/>
+      <c r="R5" s="124"/>
+      <c r="S5" s="124"/>
+      <c r="T5" s="124"/>
+      <c r="U5" s="125"/>
+      <c r="V5" s="105" t="s">
         <v>19</v>
       </c>
-      <c r="W5" s="112"/>
-      <c r="X5" s="112"/>
-      <c r="Y5" s="112"/>
-      <c r="Z5" s="112"/>
-      <c r="AA5" s="113"/>
-      <c r="AB5" s="114" t="s">
+      <c r="W5" s="106"/>
+      <c r="X5" s="106"/>
+      <c r="Y5" s="106"/>
+      <c r="Z5" s="106"/>
+      <c r="AA5" s="107"/>
+      <c r="AB5" s="108" t="s">
         <v>18</v>
       </c>
-      <c r="AC5" s="115"/>
-      <c r="AD5" s="115"/>
-      <c r="AE5" s="115"/>
-      <c r="AF5" s="115"/>
-      <c r="AG5" s="116"/>
-      <c r="AH5" s="114" t="s">
+      <c r="AC5" s="109"/>
+      <c r="AD5" s="109"/>
+      <c r="AE5" s="109"/>
+      <c r="AF5" s="109"/>
+      <c r="AG5" s="110"/>
+      <c r="AH5" s="108" t="s">
         <v>26</v>
       </c>
-      <c r="AI5" s="115"/>
-      <c r="AJ5" s="115"/>
-      <c r="AK5" s="115"/>
-      <c r="AL5" s="115"/>
-      <c r="AM5" s="116"/>
-      <c r="AN5" s="114" t="s">
+      <c r="AI5" s="109"/>
+      <c r="AJ5" s="109"/>
+      <c r="AK5" s="109"/>
+      <c r="AL5" s="109"/>
+      <c r="AM5" s="110"/>
+      <c r="AN5" s="108" t="s">
         <v>27</v>
       </c>
-      <c r="AO5" s="115"/>
-      <c r="AP5" s="115"/>
-      <c r="AQ5" s="115"/>
-      <c r="AR5" s="115"/>
-      <c r="AS5" s="116"/>
-      <c r="AT5" s="114" t="s">
+      <c r="AO5" s="109"/>
+      <c r="AP5" s="109"/>
+      <c r="AQ5" s="109"/>
+      <c r="AR5" s="109"/>
+      <c r="AS5" s="110"/>
+      <c r="AT5" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="AU5" s="115"/>
-      <c r="AV5" s="115"/>
-      <c r="AW5" s="115"/>
-      <c r="AX5" s="115"/>
-      <c r="AY5" s="116"/>
-      <c r="AZ5" s="114" t="s">
+      <c r="AU5" s="109"/>
+      <c r="AV5" s="109"/>
+      <c r="AW5" s="109"/>
+      <c r="AX5" s="109"/>
+      <c r="AY5" s="110"/>
+      <c r="AZ5" s="108" t="s">
         <v>29</v>
       </c>
-      <c r="BA5" s="115"/>
-      <c r="BB5" s="115"/>
-      <c r="BC5" s="115"/>
-      <c r="BD5" s="115"/>
-      <c r="BE5" s="116"/>
-      <c r="BF5" s="114" t="s">
+      <c r="BA5" s="109"/>
+      <c r="BB5" s="109"/>
+      <c r="BC5" s="109"/>
+      <c r="BD5" s="109"/>
+      <c r="BE5" s="110"/>
+      <c r="BF5" s="108" t="s">
         <v>30</v>
       </c>
-      <c r="BG5" s="115"/>
-      <c r="BH5" s="115"/>
-      <c r="BI5" s="115"/>
-      <c r="BJ5" s="115"/>
-      <c r="BK5" s="116"/>
-      <c r="BL5" s="96" t="s">
+      <c r="BG5" s="109"/>
+      <c r="BH5" s="109"/>
+      <c r="BI5" s="109"/>
+      <c r="BJ5" s="109"/>
+      <c r="BK5" s="110"/>
+      <c r="BL5" s="90" t="s">
         <v>31</v>
       </c>
-      <c r="BM5" s="98"/>
-      <c r="BN5" s="98"/>
-      <c r="BO5" s="99"/>
-      <c r="BP5" s="99"/>
-      <c r="BQ5" s="100"/>
+      <c r="BM5" s="92"/>
+      <c r="BN5" s="92"/>
+      <c r="BO5" s="93"/>
+      <c r="BP5" s="93"/>
+      <c r="BQ5" s="94"/>
     </row>
     <row r="6" spans="1:69" ht="103.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="110"/>
-      <c r="B6" s="95"/>
-      <c r="C6" s="90" t="s">
+      <c r="A6" s="104"/>
+      <c r="B6" s="112"/>
+      <c r="C6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="91"/>
-      <c r="E6" s="90" t="s">
+      <c r="D6" s="129"/>
+      <c r="E6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="91"/>
-      <c r="G6" s="90" t="s">
+      <c r="F6" s="129"/>
+      <c r="G6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="91"/>
-      <c r="I6" s="90" t="s">
+      <c r="H6" s="129"/>
+      <c r="I6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="J6" s="91"/>
-      <c r="K6" s="90" t="s">
+      <c r="J6" s="129"/>
+      <c r="K6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="L6" s="91"/>
-      <c r="M6" s="90" t="s">
+      <c r="L6" s="129"/>
+      <c r="M6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="N6" s="91"/>
-      <c r="O6" s="127"/>
-      <c r="P6" s="90" t="s">
+      <c r="N6" s="129"/>
+      <c r="O6" s="124"/>
+      <c r="P6" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="Q6" s="91"/>
-      <c r="R6" s="90" t="s">
+      <c r="Q6" s="129"/>
+      <c r="R6" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="S6" s="91"/>
-      <c r="T6" s="90" t="s">
+      <c r="S6" s="129"/>
+      <c r="T6" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="U6" s="91"/>
-      <c r="V6" s="95" t="s">
+      <c r="U6" s="129"/>
+      <c r="V6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="W6" s="94"/>
-      <c r="X6" s="92" t="s">
+      <c r="W6" s="127"/>
+      <c r="X6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="Y6" s="94"/>
-      <c r="Z6" s="92" t="s">
+      <c r="Y6" s="127"/>
+      <c r="Z6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AA6" s="93"/>
-      <c r="AB6" s="95" t="s">
+      <c r="AA6" s="114"/>
+      <c r="AB6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AC6" s="94"/>
-      <c r="AD6" s="92" t="s">
+      <c r="AC6" s="127"/>
+      <c r="AD6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AE6" s="94"/>
-      <c r="AF6" s="92" t="s">
+      <c r="AE6" s="127"/>
+      <c r="AF6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AG6" s="93"/>
-      <c r="AH6" s="95" t="s">
+      <c r="AG6" s="114"/>
+      <c r="AH6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AI6" s="94"/>
-      <c r="AJ6" s="92" t="s">
+      <c r="AI6" s="127"/>
+      <c r="AJ6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AK6" s="94"/>
-      <c r="AL6" s="92" t="s">
+      <c r="AK6" s="127"/>
+      <c r="AL6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AM6" s="93"/>
-      <c r="AN6" s="95" t="s">
+      <c r="AM6" s="114"/>
+      <c r="AN6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AO6" s="94"/>
-      <c r="AP6" s="92" t="s">
+      <c r="AO6" s="127"/>
+      <c r="AP6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AQ6" s="94"/>
-      <c r="AR6" s="92" t="s">
+      <c r="AQ6" s="127"/>
+      <c r="AR6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AS6" s="93"/>
-      <c r="AT6" s="95" t="s">
+      <c r="AS6" s="114"/>
+      <c r="AT6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="AU6" s="94"/>
-      <c r="AV6" s="92" t="s">
+      <c r="AU6" s="127"/>
+      <c r="AV6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="AW6" s="94"/>
-      <c r="AX6" s="92" t="s">
+      <c r="AW6" s="127"/>
+      <c r="AX6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="AY6" s="93"/>
-      <c r="AZ6" s="95" t="s">
+      <c r="AY6" s="114"/>
+      <c r="AZ6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BA6" s="94"/>
-      <c r="BB6" s="92" t="s">
+      <c r="BA6" s="127"/>
+      <c r="BB6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BC6" s="94"/>
-      <c r="BD6" s="92" t="s">
+      <c r="BC6" s="127"/>
+      <c r="BD6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BE6" s="93"/>
-      <c r="BF6" s="95" t="s">
+      <c r="BE6" s="114"/>
+      <c r="BF6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BG6" s="94"/>
-      <c r="BH6" s="92" t="s">
+      <c r="BG6" s="127"/>
+      <c r="BH6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BI6" s="94"/>
-      <c r="BJ6" s="92" t="s">
+      <c r="BI6" s="127"/>
+      <c r="BJ6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BK6" s="93"/>
-      <c r="BL6" s="95" t="s">
+      <c r="BK6" s="114"/>
+      <c r="BL6" s="112" t="s">
         <v>32</v>
       </c>
-      <c r="BM6" s="94"/>
-      <c r="BN6" s="92" t="s">
+      <c r="BM6" s="127"/>
+      <c r="BN6" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="BO6" s="94"/>
-      <c r="BP6" s="92" t="s">
+      <c r="BO6" s="127"/>
+      <c r="BP6" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="BQ6" s="93"/>
+      <c r="BQ6" s="114"/>
     </row>
     <row r="7" spans="1:69" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
@@ -10552,6 +10552,38 @@
     </row>
   </sheetData>
   <mergeCells count="48">
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="AJ6:AK6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AD6:AE6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AT6:AU6"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="AP6:AQ6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="BD6:BE6"/>
+    <mergeCell ref="BB6:BC6"/>
+    <mergeCell ref="AZ6:BA6"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AV6:AW6"/>
+    <mergeCell ref="BN6:BO6"/>
+    <mergeCell ref="BL6:BM6"/>
+    <mergeCell ref="BJ6:BK6"/>
+    <mergeCell ref="BH6:BI6"/>
+    <mergeCell ref="BF6:BG6"/>
     <mergeCell ref="I4:N5"/>
     <mergeCell ref="V4:BQ4"/>
     <mergeCell ref="A4:A6"/>
@@ -10568,38 +10600,6 @@
     <mergeCell ref="C4:H5"/>
     <mergeCell ref="P4:U5"/>
     <mergeCell ref="O4:O6"/>
-    <mergeCell ref="BN6:BO6"/>
-    <mergeCell ref="BL6:BM6"/>
-    <mergeCell ref="BJ6:BK6"/>
-    <mergeCell ref="BH6:BI6"/>
-    <mergeCell ref="BF6:BG6"/>
-    <mergeCell ref="BD6:BE6"/>
-    <mergeCell ref="BB6:BC6"/>
-    <mergeCell ref="AZ6:BA6"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AV6:AW6"/>
-    <mergeCell ref="AT6:AU6"/>
-    <mergeCell ref="AR6:AS6"/>
-    <mergeCell ref="AP6:AQ6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="AJ6:AK6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AD6:AE6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="X6:Y6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="R6:S6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="G6:H6"/>
   </mergeCells>
   <conditionalFormatting sqref="D1:D1048576 F1:F1048576 H1:H1048576 J1:J1048576 L1:L1048576 N1:N1048576 Q1:Q1048576 S1:S1048576 U1:U1048576 W1:W1048576 Y1:Y1048576 AA1:AA1048576 AC1:AC1048576 AE1:AE1048576 AG1:AG1048576 AI1:AI1048576 AK1:AK1048576 AM1:AM1048576 AO1:AO1048576 AQ1:AQ1048576 AS1:AS1048576 AU1:AU1048576 AW1:AW1048576 AY1:AY1048576 BA1:BA1048576 BC1:BC1048576 BE1:BE1048576 BG1:BG1048576 BI1:BI1048576 BK1:BK1048576 BM1:BM1048576 BO1:BO1048576 BQ1:BQ1048576">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">

</xml_diff>

<commit_message>
tmp: snapshot PEB configuration, exports and UI styling before performance isolation
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
+++ b/PROJECTS_EXCEL/tests/PersonalEventBuilder/Dependencies/test_ЕЖОС.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\tests\PersonalEventBuilder\Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D687FA9E-468F-46EA-BA8F-755C48AAE456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F16426E-5760-46C8-B4DE-5050CAA7B79A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4075,7 +4075,7 @@
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B9">
-    <cfRule type="duplicateValues" dxfId="2" priority="20823"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="20825"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>